<commit_message>
Update projections: rb_2026_combined.xlsx, qb_2026_combined.xlsx
</commit_message>
<xml_diff>
--- a/projections/qb_2026_combined.xlsx
+++ b/projections/qb_2026_combined.xlsx
@@ -604,16 +604,8 @@
       <c r="U2" t="n">
         <v>0.78</v>
       </c>
-      <c r="V2" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
-      <c r="W2" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
-      </c>
+      <c r="V2" t="inlineStr"/>
+      <c r="W2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -683,11 +675,7 @@
       <c r="U3" t="n">
         <v>8.859999999999999</v>
       </c>
-      <c r="V3" t="inlineStr">
-        <is>
-          <t>55</t>
-        </is>
-      </c>
+      <c r="V3" t="inlineStr"/>
       <c r="W3" t="inlineStr"/>
     </row>
     <row r="4">
@@ -758,11 +746,7 @@
       <c r="U4" t="n">
         <v>-2.65</v>
       </c>
-      <c r="V4" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
+      <c r="V4" t="inlineStr"/>
       <c r="W4" t="inlineStr"/>
     </row>
     <row r="5">
@@ -833,11 +817,7 @@
       <c r="U5" t="n">
         <v>6.52</v>
       </c>
-      <c r="V5" t="inlineStr">
-        <is>
-          <t>30</t>
-        </is>
-      </c>
+      <c r="V5" t="inlineStr"/>
       <c r="W5" t="inlineStr"/>
     </row>
     <row r="6">
@@ -908,11 +888,7 @@
       <c r="U6" t="n">
         <v>7.94</v>
       </c>
-      <c r="V6" t="inlineStr">
-        <is>
-          <t>40</t>
-        </is>
-      </c>
+      <c r="V6" t="inlineStr"/>
       <c r="W6" t="inlineStr"/>
     </row>
     <row r="7">
@@ -983,11 +959,7 @@
       <c r="U7" t="n">
         <v>-10.74</v>
       </c>
-      <c r="V7" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
+      <c r="V7" t="inlineStr"/>
       <c r="W7" t="inlineStr"/>
     </row>
     <row r="8">
@@ -1058,11 +1030,7 @@
       <c r="U8" t="n">
         <v>12.71</v>
       </c>
-      <c r="V8" t="inlineStr">
-        <is>
-          <t>60</t>
-        </is>
-      </c>
+      <c r="V8" t="inlineStr"/>
       <c r="W8" t="inlineStr"/>
     </row>
     <row r="9">
@@ -1133,11 +1101,7 @@
       <c r="U9" t="n">
         <v>-9.98</v>
       </c>
-      <c r="V9" t="inlineStr">
-        <is>
-          <t>30</t>
-        </is>
-      </c>
+      <c r="V9" t="inlineStr"/>
       <c r="W9" t="inlineStr"/>
     </row>
     <row r="10">
@@ -1208,11 +1172,7 @@
       <c r="U10" t="n">
         <v>12.13</v>
       </c>
-      <c r="V10" t="inlineStr">
-        <is>
-          <t>70</t>
-        </is>
-      </c>
+      <c r="V10" t="inlineStr"/>
       <c r="W10" t="inlineStr"/>
     </row>
     <row r="11">
@@ -1283,11 +1243,7 @@
       <c r="U11" t="n">
         <v>-24.31</v>
       </c>
-      <c r="V11" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
+      <c r="V11" t="inlineStr"/>
       <c r="W11" t="inlineStr"/>
     </row>
     <row r="12">
@@ -1358,11 +1314,7 @@
       <c r="U12" t="n">
         <v>-20.47</v>
       </c>
-      <c r="V12" t="inlineStr">
-        <is>
-          <t>40</t>
-        </is>
-      </c>
+      <c r="V12" t="inlineStr"/>
       <c r="W12" t="inlineStr"/>
     </row>
     <row r="13">
@@ -1433,11 +1385,7 @@
       <c r="U13" t="n">
         <v>-12.62</v>
       </c>
-      <c r="V13" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
+      <c r="V13" t="inlineStr"/>
       <c r="W13" t="inlineStr"/>
     </row>
     <row r="14">
@@ -1508,11 +1456,7 @@
       <c r="U14" t="n">
         <v>-2.47</v>
       </c>
-      <c r="V14" t="inlineStr">
-        <is>
-          <t>30</t>
-        </is>
-      </c>
+      <c r="V14" t="inlineStr"/>
       <c r="W14" t="inlineStr"/>
     </row>
     <row r="15">
@@ -1583,11 +1527,7 @@
       <c r="U15" t="n">
         <v>-31.77</v>
       </c>
-      <c r="V15" t="inlineStr">
-        <is>
-          <t>30</t>
-        </is>
-      </c>
+      <c r="V15" t="inlineStr"/>
       <c r="W15" t="inlineStr"/>
     </row>
     <row r="16">
@@ -1658,11 +1598,7 @@
       <c r="U16" t="n">
         <v>-17.79</v>
       </c>
-      <c r="V16" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
+      <c r="V16" t="inlineStr"/>
       <c r="W16" t="inlineStr"/>
     </row>
     <row r="17">
@@ -1733,11 +1669,7 @@
       <c r="U17" t="n">
         <v>-37.58</v>
       </c>
-      <c r="V17" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
+      <c r="V17" t="inlineStr"/>
       <c r="W17" t="inlineStr"/>
     </row>
     <row r="18">
@@ -1808,11 +1740,7 @@
       <c r="U18" t="n">
         <v>2.88</v>
       </c>
-      <c r="V18" t="inlineStr">
-        <is>
-          <t>40</t>
-        </is>
-      </c>
+      <c r="V18" t="inlineStr"/>
       <c r="W18" t="inlineStr"/>
     </row>
     <row r="19">
@@ -1883,11 +1811,7 @@
       <c r="U19" t="n">
         <v>-13.54</v>
       </c>
-      <c r="V19" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
+      <c r="V19" t="inlineStr"/>
       <c r="W19" t="inlineStr"/>
     </row>
     <row r="20">
@@ -1958,11 +1882,7 @@
       <c r="U20" t="n">
         <v>-26.39</v>
       </c>
-      <c r="V20" t="inlineStr">
-        <is>
-          <t>40</t>
-        </is>
-      </c>
+      <c r="V20" t="inlineStr"/>
       <c r="W20" t="inlineStr"/>
     </row>
     <row r="21">
@@ -2033,11 +1953,7 @@
       <c r="U21" t="n">
         <v>-5.14</v>
       </c>
-      <c r="V21" t="inlineStr">
-        <is>
-          <t>60</t>
-        </is>
-      </c>
+      <c r="V21" t="inlineStr"/>
       <c r="W21" t="inlineStr"/>
     </row>
     <row r="22">
@@ -2108,11 +2024,7 @@
       <c r="U22" t="n">
         <v>-6.71</v>
       </c>
-      <c r="V22" t="inlineStr">
-        <is>
-          <t>70</t>
-        </is>
-      </c>
+      <c r="V22" t="inlineStr"/>
       <c r="W22" t="inlineStr"/>
     </row>
     <row r="23">
@@ -2183,11 +2095,7 @@
       <c r="U23" t="n">
         <v>18.61</v>
       </c>
-      <c r="V23" t="inlineStr">
-        <is>
-          <t>70</t>
-        </is>
-      </c>
+      <c r="V23" t="inlineStr"/>
       <c r="W23" t="inlineStr"/>
     </row>
     <row r="24">
@@ -2258,11 +2166,7 @@
       <c r="U24" t="n">
         <v>-65.38</v>
       </c>
-      <c r="V24" t="inlineStr">
-        <is>
-          <t>80</t>
-        </is>
-      </c>
+      <c r="V24" t="inlineStr"/>
       <c r="W24" t="inlineStr"/>
     </row>
     <row r="25">
@@ -2333,11 +2237,7 @@
       <c r="U25" t="n">
         <v>0.62</v>
       </c>
-      <c r="V25" t="inlineStr">
-        <is>
-          <t>40</t>
-        </is>
-      </c>
+      <c r="V25" t="inlineStr"/>
       <c r="W25" t="inlineStr"/>
     </row>
     <row r="26">
@@ -2408,11 +2308,7 @@
       <c r="U26" t="n">
         <v>-2.59</v>
       </c>
-      <c r="V26" t="inlineStr">
-        <is>
-          <t>70</t>
-        </is>
-      </c>
+      <c r="V26" t="inlineStr"/>
       <c r="W26" t="inlineStr"/>
     </row>
     <row r="27">
@@ -2483,11 +2379,7 @@
       <c r="U27" t="n">
         <v>36.72</v>
       </c>
-      <c r="V27" t="inlineStr">
-        <is>
-          <t>40</t>
-        </is>
-      </c>
+      <c r="V27" t="inlineStr"/>
       <c r="W27" t="inlineStr"/>
     </row>
     <row r="28">
@@ -2558,11 +2450,7 @@
       <c r="U28" t="n">
         <v>6.34</v>
       </c>
-      <c r="V28" t="inlineStr">
-        <is>
-          <t>80</t>
-        </is>
-      </c>
+      <c r="V28" t="inlineStr"/>
       <c r="W28" t="inlineStr"/>
     </row>
     <row r="29">
@@ -2633,11 +2521,7 @@
       <c r="U29" t="n">
         <v>-27.55</v>
       </c>
-      <c r="V29" t="inlineStr">
-        <is>
-          <t>40</t>
-        </is>
-      </c>
+      <c r="V29" t="inlineStr"/>
       <c r="W29" t="inlineStr"/>
     </row>
     <row r="30">
@@ -2708,457 +2592,429 @@
       <c r="U30" t="n">
         <v>62.14</v>
       </c>
-      <c r="V30" t="inlineStr">
-        <is>
-          <t>70</t>
-        </is>
-      </c>
+      <c r="V30" t="inlineStr"/>
       <c r="W30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Jaxson Dart</t>
+          <t>Deshaun Watson</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>NYG</t>
+          <t>CLE</t>
         </is>
       </c>
       <c r="C31" t="n">
         <v>1</v>
       </c>
       <c r="D31" t="n">
-        <v>3614.7</v>
+        <v>3502.2</v>
       </c>
       <c r="E31" t="n">
-        <v>2112.5</v>
+        <v>1243.5</v>
       </c>
       <c r="F31" t="n">
-        <v>23.17</v>
+        <v>20.08</v>
       </c>
       <c r="G31" t="n">
-        <v>13.32</v>
+        <v>7.25</v>
       </c>
       <c r="H31" t="n">
-        <v>720</v>
+        <v>424.8</v>
       </c>
       <c r="I31" t="n">
-        <v>424</v>
+        <v>149.6</v>
       </c>
       <c r="J31" t="n">
-        <v>7.64</v>
+        <v>4.32</v>
       </c>
       <c r="K31" t="n">
-        <v>4.53</v>
+        <v>1.45</v>
       </c>
       <c r="L31" t="n">
-        <v>10.24</v>
+        <v>8.99</v>
       </c>
       <c r="M31" t="n">
-        <v>6.01</v>
+        <v>3.18</v>
       </c>
       <c r="N31" t="n">
-        <v>4.08</v>
+        <v>3.65</v>
       </c>
       <c r="O31" t="n">
-        <v>2.42</v>
+        <v>1.28</v>
       </c>
       <c r="P31" t="n">
-        <v>326.47</v>
+        <v>263.53</v>
       </c>
       <c r="Q31" t="n">
-        <v>190.5</v>
+        <v>93.48</v>
       </c>
       <c r="R31" t="n">
-        <v>136.95</v>
+        <v>60.93</v>
       </c>
       <c r="S31" t="n">
-        <v>244.23</v>
+        <v>126.21</v>
       </c>
       <c r="T31" t="n">
-        <v>278.65</v>
+        <v>91.94</v>
       </c>
       <c r="U31" t="n">
-        <v>-88.15000000000001</v>
-      </c>
-      <c r="V31" t="inlineStr">
-        <is>
-          <t>60</t>
-        </is>
-      </c>
+        <v>1.54</v>
+      </c>
+      <c r="V31" t="inlineStr"/>
       <c r="W31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Deshaun Watson</t>
+          <t>Kirk Cousins</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>CLE</t>
+          <t>LV</t>
         </is>
       </c>
       <c r="C32" t="n">
         <v>1</v>
       </c>
       <c r="D32" t="n">
-        <v>3502.2</v>
+        <v>3426.8</v>
       </c>
       <c r="E32" t="n">
-        <v>1243.5</v>
+        <v>405.1</v>
       </c>
       <c r="F32" t="n">
-        <v>20.08</v>
+        <v>26.06</v>
       </c>
       <c r="G32" t="n">
-        <v>7.25</v>
+        <v>2.87</v>
       </c>
       <c r="H32" t="n">
-        <v>424.8</v>
+        <v>62.1</v>
       </c>
       <c r="I32" t="n">
-        <v>149.6</v>
+        <v>7.2</v>
       </c>
       <c r="J32" t="n">
-        <v>4.32</v>
+        <v>1.69</v>
       </c>
       <c r="K32" t="n">
-        <v>1.45</v>
+        <v>0.22</v>
       </c>
       <c r="L32" t="n">
-        <v>8.99</v>
+        <v>11.88</v>
       </c>
       <c r="M32" t="n">
-        <v>3.18</v>
+        <v>1.4</v>
       </c>
       <c r="N32" t="n">
-        <v>3.65</v>
+        <v>2.68</v>
       </c>
       <c r="O32" t="n">
-        <v>1.28</v>
+        <v>0.3</v>
       </c>
       <c r="P32" t="n">
-        <v>263.53</v>
+        <v>228.54</v>
       </c>
       <c r="Q32" t="n">
-        <v>93.48</v>
+        <v>26.32</v>
       </c>
       <c r="R32" t="n">
-        <v>60.93</v>
+        <v>17.1</v>
       </c>
       <c r="S32" t="n">
-        <v>126.21</v>
+        <v>36.88</v>
       </c>
       <c r="T32" t="n">
-        <v>91.94</v>
+        <v>43.68</v>
       </c>
       <c r="U32" t="n">
-        <v>1.54</v>
-      </c>
-      <c r="V32" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
+        <v>-17.36</v>
+      </c>
+      <c r="V32" t="inlineStr"/>
       <c r="W32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Kirk Cousins</t>
+          <t>Jaxson Dart</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>LV</t>
+          <t>NYG</t>
         </is>
       </c>
       <c r="C33" t="n">
         <v>1</v>
       </c>
       <c r="D33" t="n">
-        <v>3426.8</v>
+        <v>3614.7</v>
       </c>
       <c r="E33" t="n">
-        <v>405.1</v>
+        <v>213.7</v>
       </c>
       <c r="F33" t="n">
-        <v>26.06</v>
+        <v>23.17</v>
       </c>
       <c r="G33" t="n">
-        <v>2.87</v>
+        <v>1.44</v>
       </c>
       <c r="H33" t="n">
-        <v>62.1</v>
+        <v>720</v>
       </c>
       <c r="I33" t="n">
-        <v>7.2</v>
+        <v>42.4</v>
       </c>
       <c r="J33" t="n">
-        <v>1.69</v>
+        <v>7.64</v>
       </c>
       <c r="K33" t="n">
-        <v>0.22</v>
+        <v>0.44</v>
       </c>
       <c r="L33" t="n">
-        <v>11.88</v>
+        <v>10.24</v>
       </c>
       <c r="M33" t="n">
-        <v>1.4</v>
+        <v>0.6</v>
       </c>
       <c r="N33" t="n">
-        <v>2.68</v>
+        <v>4.08</v>
       </c>
       <c r="O33" t="n">
-        <v>0.3</v>
+        <v>0.23</v>
       </c>
       <c r="P33" t="n">
-        <v>228.54</v>
+        <v>326.47</v>
       </c>
       <c r="Q33" t="n">
-        <v>26.32</v>
+        <v>19.53</v>
       </c>
       <c r="R33" t="n">
-        <v>17.1</v>
+        <v>14.04</v>
       </c>
       <c r="S33" t="n">
-        <v>36.88</v>
+        <v>25.04</v>
       </c>
       <c r="T33" t="n">
-        <v>43.68</v>
+        <v>278.65</v>
       </c>
       <c r="U33" t="n">
-        <v>-17.36</v>
-      </c>
-      <c r="V33" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
+        <v>-259.12</v>
+      </c>
+      <c r="V33" t="inlineStr"/>
       <c r="W33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Fernando Mendoza</t>
+          <t>Jameis Winston</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>LV</t>
+          <t>NYG</t>
         </is>
       </c>
       <c r="C34" t="n">
         <v>2</v>
       </c>
       <c r="D34" t="n">
-        <v>3779.2</v>
+        <v>3385.3</v>
       </c>
       <c r="E34" t="n">
-        <v>2870.1</v>
+        <v>2774.6</v>
       </c>
       <c r="F34" t="n">
-        <v>17.12</v>
+        <v>23.03</v>
       </c>
       <c r="G34" t="n">
-        <v>13.07</v>
+        <v>18.79</v>
       </c>
       <c r="H34" t="n">
-        <v>223.3</v>
+        <v>188.9</v>
       </c>
       <c r="I34" t="n">
-        <v>171.1</v>
+        <v>155.8</v>
       </c>
       <c r="J34" t="n">
-        <v>3.89</v>
+        <v>2.33</v>
       </c>
       <c r="K34" t="n">
-        <v>2.94</v>
+        <v>1.93</v>
       </c>
       <c r="L34" t="n">
-        <v>12.73</v>
+        <v>15.13</v>
       </c>
       <c r="M34" t="n">
-        <v>9.73</v>
+        <v>12.45</v>
       </c>
       <c r="N34" t="n">
-        <v>2.72</v>
+        <v>3.4</v>
       </c>
       <c r="O34" t="n">
-        <v>2.07</v>
+        <v>2.8</v>
       </c>
       <c r="P34" t="n">
-        <v>234.42</v>
+        <v>223.34</v>
       </c>
       <c r="Q34" t="n">
-        <v>178.23</v>
+        <v>182.8</v>
       </c>
       <c r="R34" t="n">
-        <v>108.07</v>
+        <v>108.53</v>
       </c>
       <c r="S34" t="n">
-        <v>247.88</v>
-      </c>
-      <c r="T34" t="n">
-        <v>170.12</v>
-      </c>
-      <c r="U34" t="n">
-        <v>8.109999999999999</v>
-      </c>
-      <c r="V34" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
+        <v>258.17</v>
+      </c>
+      <c r="T34" t="inlineStr"/>
+      <c r="U34" t="inlineStr"/>
+      <c r="V34" t="inlineStr"/>
       <c r="W34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Shedeur Sanders</t>
+          <t>Fernando Mendoza</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>CLE</t>
+          <t>LV</t>
         </is>
       </c>
       <c r="C35" t="n">
         <v>2</v>
       </c>
       <c r="D35" t="n">
-        <v>3400.9</v>
+        <v>3779.2</v>
       </c>
       <c r="E35" t="n">
-        <v>1792.6</v>
+        <v>2870.1</v>
       </c>
       <c r="F35" t="n">
-        <v>16.16</v>
+        <v>17.12</v>
       </c>
       <c r="G35" t="n">
-        <v>8.529999999999999</v>
+        <v>13.07</v>
       </c>
       <c r="H35" t="n">
-        <v>282.1</v>
+        <v>223.3</v>
       </c>
       <c r="I35" t="n">
-        <v>150.4</v>
+        <v>171.1</v>
       </c>
       <c r="J35" t="n">
-        <v>2.89</v>
+        <v>3.89</v>
       </c>
       <c r="K35" t="n">
-        <v>1.56</v>
+        <v>2.94</v>
       </c>
       <c r="L35" t="n">
-        <v>12.11</v>
+        <v>12.73</v>
       </c>
       <c r="M35" t="n">
-        <v>6.4</v>
+        <v>9.73</v>
       </c>
       <c r="N35" t="n">
-        <v>4.97</v>
+        <v>2.72</v>
       </c>
       <c r="O35" t="n">
-        <v>2.65</v>
+        <v>2.07</v>
       </c>
       <c r="P35" t="n">
-        <v>212.07</v>
+        <v>234.42</v>
       </c>
       <c r="Q35" t="n">
-        <v>112.12</v>
+        <v>178.23</v>
       </c>
       <c r="R35" t="n">
-        <v>63.43</v>
+        <v>108.07</v>
       </c>
       <c r="S35" t="n">
-        <v>160.74</v>
+        <v>247.88</v>
       </c>
       <c r="T35" t="n">
-        <v>92.91</v>
+        <v>170.12</v>
       </c>
       <c r="U35" t="n">
-        <v>19.21</v>
-      </c>
-      <c r="V35" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
+        <v>8.109999999999999</v>
+      </c>
+      <c r="V35" t="inlineStr"/>
       <c r="W35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Jameis Winston</t>
+          <t>Shedeur Sanders</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>NYG</t>
+          <t>CLE</t>
         </is>
       </c>
       <c r="C36" t="n">
         <v>2</v>
       </c>
       <c r="D36" t="n">
-        <v>3385.3</v>
+        <v>3400.9</v>
       </c>
       <c r="E36" t="n">
-        <v>997.2</v>
+        <v>1792.6</v>
       </c>
       <c r="F36" t="n">
-        <v>23.03</v>
+        <v>16.16</v>
       </c>
       <c r="G36" t="n">
-        <v>6.88</v>
+        <v>8.529999999999999</v>
       </c>
       <c r="H36" t="n">
-        <v>188.9</v>
+        <v>282.1</v>
       </c>
       <c r="I36" t="n">
-        <v>55.3</v>
+        <v>150.4</v>
       </c>
       <c r="J36" t="n">
-        <v>2.33</v>
+        <v>2.89</v>
       </c>
       <c r="K36" t="n">
-        <v>0.6899999999999999</v>
+        <v>1.56</v>
       </c>
       <c r="L36" t="n">
-        <v>15.13</v>
+        <v>12.11</v>
       </c>
       <c r="M36" t="n">
-        <v>4.46</v>
+        <v>6.4</v>
       </c>
       <c r="N36" t="n">
-        <v>3.4</v>
+        <v>4.97</v>
       </c>
       <c r="O36" t="n">
-        <v>1</v>
+        <v>2.65</v>
       </c>
       <c r="P36" t="n">
-        <v>223.34</v>
+        <v>212.07</v>
       </c>
       <c r="Q36" t="n">
-        <v>66.16</v>
+        <v>112.12</v>
       </c>
       <c r="R36" t="n">
-        <v>39.28</v>
+        <v>63.43</v>
       </c>
       <c r="S36" t="n">
-        <v>93.44</v>
-      </c>
-      <c r="T36" t="inlineStr"/>
-      <c r="U36" t="inlineStr"/>
-      <c r="V36" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
+        <v>160.74</v>
+      </c>
+      <c r="T36" t="n">
+        <v>92.91</v>
+      </c>
+      <c r="U36" t="n">
+        <v>19.21</v>
+      </c>
+      <c r="V36" t="inlineStr"/>
       <c r="W36" t="inlineStr"/>
     </row>
     <row r="37">
@@ -3225,11 +3081,7 @@
       </c>
       <c r="T37" t="inlineStr"/>
       <c r="U37" t="inlineStr"/>
-      <c r="V37" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
+      <c r="V37" t="inlineStr"/>
       <c r="W37" t="inlineStr"/>
     </row>
     <row r="38">
@@ -3296,11 +3148,7 @@
       </c>
       <c r="T38" t="inlineStr"/>
       <c r="U38" t="inlineStr"/>
-      <c r="V38" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
+      <c r="V38" t="inlineStr"/>
       <c r="W38" t="inlineStr"/>
     </row>
     <row r="39">
@@ -3367,11 +3215,7 @@
       </c>
       <c r="T39" t="inlineStr"/>
       <c r="U39" t="inlineStr"/>
-      <c r="V39" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
+      <c r="V39" t="inlineStr"/>
       <c r="W39" t="inlineStr"/>
     </row>
     <row r="40">
@@ -3442,11 +3286,7 @@
       <c r="U40" t="n">
         <v>-21.18</v>
       </c>
-      <c r="V40" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
+      <c r="V40" t="inlineStr"/>
       <c r="W40" t="inlineStr"/>
     </row>
     <row r="41">
@@ -3580,11 +3420,7 @@
       </c>
       <c r="T42" t="inlineStr"/>
       <c r="U42" t="inlineStr"/>
-      <c r="V42" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
+      <c r="V42" t="inlineStr"/>
       <c r="W42" t="inlineStr"/>
     </row>
     <row r="43">
@@ -3651,11 +3487,7 @@
       </c>
       <c r="T43" t="inlineStr"/>
       <c r="U43" t="inlineStr"/>
-      <c r="V43" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
+      <c r="V43" t="inlineStr"/>
       <c r="W43" t="inlineStr"/>
     </row>
     <row r="44">
@@ -3722,11 +3554,7 @@
       </c>
       <c r="T44" t="inlineStr"/>
       <c r="U44" t="inlineStr"/>
-      <c r="V44" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
+      <c r="V44" t="inlineStr"/>
       <c r="W44" t="inlineStr"/>
     </row>
     <row r="45">
@@ -3860,11 +3688,7 @@
       </c>
       <c r="T46" t="inlineStr"/>
       <c r="U46" t="inlineStr"/>
-      <c r="V46" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
+      <c r="V46" t="inlineStr"/>
       <c r="W46" t="inlineStr"/>
     </row>
     <row r="47">
@@ -3931,11 +3755,7 @@
       </c>
       <c r="T47" t="inlineStr"/>
       <c r="U47" t="inlineStr"/>
-      <c r="V47" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
+      <c r="V47" t="inlineStr"/>
       <c r="W47" t="inlineStr"/>
     </row>
     <row r="48">
@@ -4069,11 +3889,7 @@
       </c>
       <c r="T49" t="inlineStr"/>
       <c r="U49" t="inlineStr"/>
-      <c r="V49" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
+      <c r="V49" t="inlineStr"/>
       <c r="W49" t="inlineStr"/>
     </row>
     <row r="50">
@@ -4140,11 +3956,7 @@
       </c>
       <c r="T50" t="inlineStr"/>
       <c r="U50" t="inlineStr"/>
-      <c r="V50" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
+      <c r="V50" t="inlineStr"/>
       <c r="W50" t="inlineStr"/>
     </row>
     <row r="51">
@@ -4211,11 +4023,7 @@
       </c>
       <c r="T51" t="inlineStr"/>
       <c r="U51" t="inlineStr"/>
-      <c r="V51" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
+      <c r="V51" t="inlineStr"/>
       <c r="W51" t="inlineStr"/>
     </row>
     <row r="52">
@@ -4349,11 +4157,7 @@
       </c>
       <c r="T53" t="inlineStr"/>
       <c r="U53" t="inlineStr"/>
-      <c r="V53" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
+      <c r="V53" t="inlineStr"/>
       <c r="W53" t="inlineStr"/>
     </row>
     <row r="54">
@@ -4420,11 +4224,7 @@
       </c>
       <c r="T54" t="inlineStr"/>
       <c r="U54" t="inlineStr"/>
-      <c r="V54" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
+      <c r="V54" t="inlineStr"/>
       <c r="W54" t="inlineStr"/>
     </row>
     <row r="55">
@@ -4491,11 +4291,7 @@
       </c>
       <c r="T55" t="inlineStr"/>
       <c r="U55" t="inlineStr"/>
-      <c r="V55" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
+      <c r="V55" t="inlineStr"/>
       <c r="W55" t="inlineStr"/>
     </row>
     <row r="56">
@@ -4562,11 +4358,7 @@
       </c>
       <c r="T56" t="inlineStr"/>
       <c r="U56" t="inlineStr"/>
-      <c r="V56" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
+      <c r="V56" t="inlineStr"/>
       <c r="W56" t="inlineStr"/>
     </row>
     <row r="57">
@@ -4700,11 +4492,7 @@
       </c>
       <c r="T58" t="inlineStr"/>
       <c r="U58" t="inlineStr"/>
-      <c r="V58" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
+      <c r="V58" t="inlineStr"/>
       <c r="W58" t="inlineStr"/>
     </row>
     <row r="59">
@@ -4838,11 +4626,7 @@
       </c>
       <c r="T60" t="inlineStr"/>
       <c r="U60" t="inlineStr"/>
-      <c r="V60" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
+      <c r="V60" t="inlineStr"/>
       <c r="W60" t="inlineStr"/>
     </row>
     <row r="61">
@@ -4909,11 +4693,7 @@
       </c>
       <c r="T61" t="inlineStr"/>
       <c r="U61" t="inlineStr"/>
-      <c r="V61" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
+      <c r="V61" t="inlineStr"/>
       <c r="W61" t="inlineStr"/>
     </row>
     <row r="62">
@@ -4984,11 +4764,7 @@
       <c r="U62" t="n">
         <v>-71.12</v>
       </c>
-      <c r="V62" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
+      <c r="V62" t="inlineStr"/>
       <c r="W62" t="inlineStr"/>
     </row>
     <row r="63">
@@ -5055,11 +4831,7 @@
       </c>
       <c r="T63" t="inlineStr"/>
       <c r="U63" t="inlineStr"/>
-      <c r="V63" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
+      <c r="V63" t="inlineStr"/>
       <c r="W63" t="inlineStr"/>
     </row>
     <row r="64">
@@ -5126,11 +4898,7 @@
       </c>
       <c r="T64" t="inlineStr"/>
       <c r="U64" t="inlineStr"/>
-      <c r="V64" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
+      <c r="V64" t="inlineStr"/>
       <c r="W64" t="inlineStr"/>
     </row>
     <row r="65">
@@ -5197,11 +4965,7 @@
       </c>
       <c r="T65" t="inlineStr"/>
       <c r="U65" t="inlineStr"/>
-      <c r="V65" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
+      <c r="V65" t="inlineStr"/>
       <c r="W65" t="inlineStr"/>
     </row>
   </sheetData>
@@ -5403,16 +5167,8 @@
       <c r="U2" t="n">
         <v>0.78</v>
       </c>
-      <c r="V2" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
-      <c r="W2" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
-      </c>
+      <c r="V2" t="inlineStr"/>
+      <c r="W2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -5482,11 +5238,7 @@
       <c r="U3" t="n">
         <v>8.859999999999999</v>
       </c>
-      <c r="V3" t="inlineStr">
-        <is>
-          <t>55</t>
-        </is>
-      </c>
+      <c r="V3" t="inlineStr"/>
       <c r="W3" t="inlineStr"/>
     </row>
     <row r="4">
@@ -5557,11 +5309,7 @@
       <c r="U4" t="n">
         <v>-2.65</v>
       </c>
-      <c r="V4" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
+      <c r="V4" t="inlineStr"/>
       <c r="W4" t="inlineStr"/>
     </row>
     <row r="5">
@@ -5632,11 +5380,7 @@
       <c r="U5" t="n">
         <v>6.52</v>
       </c>
-      <c r="V5" t="inlineStr">
-        <is>
-          <t>30</t>
-        </is>
-      </c>
+      <c r="V5" t="inlineStr"/>
       <c r="W5" t="inlineStr"/>
     </row>
     <row r="6">
@@ -5707,11 +5451,7 @@
       <c r="U6" t="n">
         <v>7.94</v>
       </c>
-      <c r="V6" t="inlineStr">
-        <is>
-          <t>40</t>
-        </is>
-      </c>
+      <c r="V6" t="inlineStr"/>
       <c r="W6" t="inlineStr"/>
     </row>
     <row r="7">
@@ -5782,11 +5522,7 @@
       <c r="U7" t="n">
         <v>-10.74</v>
       </c>
-      <c r="V7" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
+      <c r="V7" t="inlineStr"/>
       <c r="W7" t="inlineStr"/>
     </row>
     <row r="8">
@@ -5857,11 +5593,7 @@
       <c r="U8" t="n">
         <v>12.71</v>
       </c>
-      <c r="V8" t="inlineStr">
-        <is>
-          <t>60</t>
-        </is>
-      </c>
+      <c r="V8" t="inlineStr"/>
       <c r="W8" t="inlineStr"/>
     </row>
     <row r="9">
@@ -5932,11 +5664,7 @@
       <c r="U9" t="n">
         <v>-9.98</v>
       </c>
-      <c r="V9" t="inlineStr">
-        <is>
-          <t>30</t>
-        </is>
-      </c>
+      <c r="V9" t="inlineStr"/>
       <c r="W9" t="inlineStr"/>
     </row>
     <row r="10">
@@ -6007,11 +5735,7 @@
       <c r="U10" t="n">
         <v>12.13</v>
       </c>
-      <c r="V10" t="inlineStr">
-        <is>
-          <t>70</t>
-        </is>
-      </c>
+      <c r="V10" t="inlineStr"/>
       <c r="W10" t="inlineStr"/>
     </row>
     <row r="11">
@@ -6082,11 +5806,7 @@
       <c r="U11" t="n">
         <v>-24.31</v>
       </c>
-      <c r="V11" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
+      <c r="V11" t="inlineStr"/>
       <c r="W11" t="inlineStr"/>
     </row>
     <row r="12">
@@ -6157,11 +5877,7 @@
       <c r="U12" t="n">
         <v>-20.47</v>
       </c>
-      <c r="V12" t="inlineStr">
-        <is>
-          <t>40</t>
-        </is>
-      </c>
+      <c r="V12" t="inlineStr"/>
       <c r="W12" t="inlineStr"/>
     </row>
     <row r="13">
@@ -6232,11 +5948,7 @@
       <c r="U13" t="n">
         <v>-12.62</v>
       </c>
-      <c r="V13" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
+      <c r="V13" t="inlineStr"/>
       <c r="W13" t="inlineStr"/>
     </row>
     <row r="14">
@@ -6307,11 +6019,7 @@
       <c r="U14" t="n">
         <v>-2.47</v>
       </c>
-      <c r="V14" t="inlineStr">
-        <is>
-          <t>30</t>
-        </is>
-      </c>
+      <c r="V14" t="inlineStr"/>
       <c r="W14" t="inlineStr"/>
     </row>
     <row r="15">
@@ -6382,11 +6090,7 @@
       <c r="U15" t="n">
         <v>-31.77</v>
       </c>
-      <c r="V15" t="inlineStr">
-        <is>
-          <t>30</t>
-        </is>
-      </c>
+      <c r="V15" t="inlineStr"/>
       <c r="W15" t="inlineStr"/>
     </row>
     <row r="16">
@@ -6457,11 +6161,7 @@
       <c r="U16" t="n">
         <v>-17.79</v>
       </c>
-      <c r="V16" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
+      <c r="V16" t="inlineStr"/>
       <c r="W16" t="inlineStr"/>
     </row>
     <row r="17">
@@ -6532,11 +6232,7 @@
       <c r="U17" t="n">
         <v>-37.58</v>
       </c>
-      <c r="V17" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
+      <c r="V17" t="inlineStr"/>
       <c r="W17" t="inlineStr"/>
     </row>
     <row r="18">
@@ -6607,11 +6303,7 @@
       <c r="U18" t="n">
         <v>2.88</v>
       </c>
-      <c r="V18" t="inlineStr">
-        <is>
-          <t>40</t>
-        </is>
-      </c>
+      <c r="V18" t="inlineStr"/>
       <c r="W18" t="inlineStr"/>
     </row>
     <row r="19">
@@ -6682,11 +6374,7 @@
       <c r="U19" t="n">
         <v>-13.54</v>
       </c>
-      <c r="V19" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
+      <c r="V19" t="inlineStr"/>
       <c r="W19" t="inlineStr"/>
     </row>
     <row r="20">
@@ -6757,11 +6445,7 @@
       <c r="U20" t="n">
         <v>-26.39</v>
       </c>
-      <c r="V20" t="inlineStr">
-        <is>
-          <t>40</t>
-        </is>
-      </c>
+      <c r="V20" t="inlineStr"/>
       <c r="W20" t="inlineStr"/>
     </row>
     <row r="21">
@@ -6832,11 +6516,7 @@
       <c r="U21" t="n">
         <v>-5.14</v>
       </c>
-      <c r="V21" t="inlineStr">
-        <is>
-          <t>60</t>
-        </is>
-      </c>
+      <c r="V21" t="inlineStr"/>
       <c r="W21" t="inlineStr"/>
     </row>
     <row r="22">
@@ -6907,11 +6587,7 @@
       <c r="U22" t="n">
         <v>-6.71</v>
       </c>
-      <c r="V22" t="inlineStr">
-        <is>
-          <t>70</t>
-        </is>
-      </c>
+      <c r="V22" t="inlineStr"/>
       <c r="W22" t="inlineStr"/>
     </row>
     <row r="23">
@@ -6982,11 +6658,7 @@
       <c r="U23" t="n">
         <v>18.61</v>
       </c>
-      <c r="V23" t="inlineStr">
-        <is>
-          <t>70</t>
-        </is>
-      </c>
+      <c r="V23" t="inlineStr"/>
       <c r="W23" t="inlineStr"/>
     </row>
     <row r="24">
@@ -7057,11 +6729,7 @@
       <c r="U24" t="n">
         <v>-65.38</v>
       </c>
-      <c r="V24" t="inlineStr">
-        <is>
-          <t>80</t>
-        </is>
-      </c>
+      <c r="V24" t="inlineStr"/>
       <c r="W24" t="inlineStr"/>
     </row>
     <row r="25">
@@ -7132,11 +6800,7 @@
       <c r="U25" t="n">
         <v>0.62</v>
       </c>
-      <c r="V25" t="inlineStr">
-        <is>
-          <t>40</t>
-        </is>
-      </c>
+      <c r="V25" t="inlineStr"/>
       <c r="W25" t="inlineStr"/>
     </row>
     <row r="26">
@@ -7207,11 +6871,7 @@
       <c r="U26" t="n">
         <v>-2.59</v>
       </c>
-      <c r="V26" t="inlineStr">
-        <is>
-          <t>70</t>
-        </is>
-      </c>
+      <c r="V26" t="inlineStr"/>
       <c r="W26" t="inlineStr"/>
     </row>
     <row r="27">
@@ -7282,11 +6942,7 @@
       <c r="U27" t="n">
         <v>36.72</v>
       </c>
-      <c r="V27" t="inlineStr">
-        <is>
-          <t>40</t>
-        </is>
-      </c>
+      <c r="V27" t="inlineStr"/>
       <c r="W27" t="inlineStr"/>
     </row>
     <row r="28">
@@ -7357,11 +7013,7 @@
       <c r="U28" t="n">
         <v>6.34</v>
       </c>
-      <c r="V28" t="inlineStr">
-        <is>
-          <t>80</t>
-        </is>
-      </c>
+      <c r="V28" t="inlineStr"/>
       <c r="W28" t="inlineStr"/>
     </row>
     <row r="29">
@@ -7432,11 +7084,7 @@
       <c r="U29" t="n">
         <v>-27.55</v>
       </c>
-      <c r="V29" t="inlineStr">
-        <is>
-          <t>40</t>
-        </is>
-      </c>
+      <c r="V29" t="inlineStr"/>
       <c r="W29" t="inlineStr"/>
     </row>
     <row r="30">
@@ -7507,236 +7155,220 @@
       <c r="U30" t="n">
         <v>62.14</v>
       </c>
-      <c r="V30" t="inlineStr">
-        <is>
-          <t>70</t>
-        </is>
-      </c>
+      <c r="V30" t="inlineStr"/>
       <c r="W30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Jaxson Dart</t>
+          <t>Deshaun Watson</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>NYG</t>
+          <t>CLE</t>
         </is>
       </c>
       <c r="C31" t="n">
         <v>1</v>
       </c>
       <c r="D31" t="n">
-        <v>3614.7</v>
+        <v>3502.2</v>
       </c>
       <c r="E31" t="n">
-        <v>2112.5</v>
+        <v>1243.5</v>
       </c>
       <c r="F31" t="n">
-        <v>23.17</v>
+        <v>20.08</v>
       </c>
       <c r="G31" t="n">
-        <v>13.32</v>
+        <v>7.25</v>
       </c>
       <c r="H31" t="n">
-        <v>720</v>
+        <v>424.8</v>
       </c>
       <c r="I31" t="n">
-        <v>424</v>
+        <v>149.6</v>
       </c>
       <c r="J31" t="n">
-        <v>7.64</v>
+        <v>4.32</v>
       </c>
       <c r="K31" t="n">
-        <v>4.53</v>
+        <v>1.45</v>
       </c>
       <c r="L31" t="n">
-        <v>10.24</v>
+        <v>8.99</v>
       </c>
       <c r="M31" t="n">
-        <v>6.01</v>
+        <v>3.18</v>
       </c>
       <c r="N31" t="n">
-        <v>4.08</v>
+        <v>3.65</v>
       </c>
       <c r="O31" t="n">
-        <v>2.42</v>
+        <v>1.28</v>
       </c>
       <c r="P31" t="n">
-        <v>326.47</v>
+        <v>263.53</v>
       </c>
       <c r="Q31" t="n">
-        <v>190.5</v>
+        <v>93.48</v>
       </c>
       <c r="R31" t="n">
-        <v>136.95</v>
+        <v>60.93</v>
       </c>
       <c r="S31" t="n">
-        <v>244.23</v>
+        <v>126.21</v>
       </c>
       <c r="T31" t="n">
-        <v>278.65</v>
+        <v>91.94</v>
       </c>
       <c r="U31" t="n">
-        <v>-88.15000000000001</v>
-      </c>
-      <c r="V31" t="inlineStr">
-        <is>
-          <t>60</t>
-        </is>
-      </c>
+        <v>1.54</v>
+      </c>
+      <c r="V31" t="inlineStr"/>
       <c r="W31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Deshaun Watson</t>
+          <t>Kirk Cousins</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>CLE</t>
+          <t>LV</t>
         </is>
       </c>
       <c r="C32" t="n">
         <v>1</v>
       </c>
       <c r="D32" t="n">
-        <v>3502.2</v>
+        <v>3426.8</v>
       </c>
       <c r="E32" t="n">
-        <v>1243.5</v>
+        <v>405.1</v>
       </c>
       <c r="F32" t="n">
-        <v>20.08</v>
+        <v>26.06</v>
       </c>
       <c r="G32" t="n">
-        <v>7.25</v>
+        <v>2.87</v>
       </c>
       <c r="H32" t="n">
-        <v>424.8</v>
+        <v>62.1</v>
       </c>
       <c r="I32" t="n">
-        <v>149.6</v>
+        <v>7.2</v>
       </c>
       <c r="J32" t="n">
-        <v>4.32</v>
+        <v>1.69</v>
       </c>
       <c r="K32" t="n">
-        <v>1.45</v>
+        <v>0.22</v>
       </c>
       <c r="L32" t="n">
-        <v>8.99</v>
+        <v>11.88</v>
       </c>
       <c r="M32" t="n">
-        <v>3.18</v>
+        <v>1.4</v>
       </c>
       <c r="N32" t="n">
-        <v>3.65</v>
+        <v>2.68</v>
       </c>
       <c r="O32" t="n">
-        <v>1.28</v>
+        <v>0.3</v>
       </c>
       <c r="P32" t="n">
-        <v>263.53</v>
+        <v>228.54</v>
       </c>
       <c r="Q32" t="n">
-        <v>93.48</v>
+        <v>26.32</v>
       </c>
       <c r="R32" t="n">
-        <v>60.93</v>
+        <v>17.1</v>
       </c>
       <c r="S32" t="n">
-        <v>126.21</v>
+        <v>36.88</v>
       </c>
       <c r="T32" t="n">
-        <v>91.94</v>
+        <v>43.68</v>
       </c>
       <c r="U32" t="n">
-        <v>1.54</v>
-      </c>
-      <c r="V32" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
+        <v>-17.36</v>
+      </c>
+      <c r="V32" t="inlineStr"/>
       <c r="W32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Kirk Cousins</t>
+          <t>Jaxson Dart</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>LV</t>
+          <t>NYG</t>
         </is>
       </c>
       <c r="C33" t="n">
         <v>1</v>
       </c>
       <c r="D33" t="n">
-        <v>3426.8</v>
+        <v>3614.7</v>
       </c>
       <c r="E33" t="n">
-        <v>405.1</v>
+        <v>213.7</v>
       </c>
       <c r="F33" t="n">
-        <v>26.06</v>
+        <v>23.17</v>
       </c>
       <c r="G33" t="n">
-        <v>2.87</v>
+        <v>1.44</v>
       </c>
       <c r="H33" t="n">
-        <v>62.1</v>
+        <v>720</v>
       </c>
       <c r="I33" t="n">
-        <v>7.2</v>
+        <v>42.4</v>
       </c>
       <c r="J33" t="n">
-        <v>1.69</v>
+        <v>7.64</v>
       </c>
       <c r="K33" t="n">
-        <v>0.22</v>
+        <v>0.44</v>
       </c>
       <c r="L33" t="n">
-        <v>11.88</v>
+        <v>10.24</v>
       </c>
       <c r="M33" t="n">
-        <v>1.4</v>
+        <v>0.6</v>
       </c>
       <c r="N33" t="n">
-        <v>2.68</v>
+        <v>4.08</v>
       </c>
       <c r="O33" t="n">
-        <v>0.3</v>
+        <v>0.23</v>
       </c>
       <c r="P33" t="n">
-        <v>228.54</v>
+        <v>326.47</v>
       </c>
       <c r="Q33" t="n">
-        <v>26.32</v>
+        <v>19.53</v>
       </c>
       <c r="R33" t="n">
-        <v>17.1</v>
+        <v>14.04</v>
       </c>
       <c r="S33" t="n">
-        <v>36.88</v>
+        <v>25.04</v>
       </c>
       <c r="T33" t="n">
-        <v>43.68</v>
+        <v>278.65</v>
       </c>
       <c r="U33" t="n">
-        <v>-17.36</v>
-      </c>
-      <c r="V33" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
+        <v>-259.12</v>
+      </c>
+      <c r="V33" t="inlineStr"/>
       <c r="W33" t="inlineStr"/>
     </row>
   </sheetData>
@@ -7873,222 +7505,210 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Fernando Mendoza</t>
+          <t>Jameis Winston</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>LV</t>
+          <t>NYG</t>
         </is>
       </c>
       <c r="C2" t="n">
         <v>2</v>
       </c>
       <c r="D2" t="n">
-        <v>3779.2</v>
+        <v>3385.3</v>
       </c>
       <c r="E2" t="n">
-        <v>2870.1</v>
+        <v>2774.6</v>
       </c>
       <c r="F2" t="n">
-        <v>17.12</v>
+        <v>23.03</v>
       </c>
       <c r="G2" t="n">
-        <v>13.07</v>
+        <v>18.79</v>
       </c>
       <c r="H2" t="n">
-        <v>223.3</v>
+        <v>188.9</v>
       </c>
       <c r="I2" t="n">
-        <v>171.1</v>
+        <v>155.8</v>
       </c>
       <c r="J2" t="n">
-        <v>3.89</v>
+        <v>2.33</v>
       </c>
       <c r="K2" t="n">
-        <v>2.94</v>
+        <v>1.93</v>
       </c>
       <c r="L2" t="n">
-        <v>12.73</v>
+        <v>15.13</v>
       </c>
       <c r="M2" t="n">
-        <v>9.73</v>
+        <v>12.45</v>
       </c>
       <c r="N2" t="n">
-        <v>2.72</v>
+        <v>3.4</v>
       </c>
       <c r="O2" t="n">
-        <v>2.07</v>
+        <v>2.8</v>
       </c>
       <c r="P2" t="n">
-        <v>234.42</v>
+        <v>223.34</v>
       </c>
       <c r="Q2" t="n">
-        <v>178.23</v>
+        <v>182.8</v>
       </c>
       <c r="R2" t="n">
-        <v>108.07</v>
+        <v>108.53</v>
       </c>
       <c r="S2" t="n">
-        <v>247.88</v>
-      </c>
-      <c r="T2" t="n">
-        <v>170.12</v>
-      </c>
-      <c r="U2" t="n">
-        <v>8.109999999999999</v>
-      </c>
-      <c r="V2" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
+        <v>258.17</v>
+      </c>
+      <c r="T2" t="inlineStr"/>
+      <c r="U2" t="inlineStr"/>
+      <c r="V2" t="inlineStr"/>
       <c r="W2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Shedeur Sanders</t>
+          <t>Fernando Mendoza</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>CLE</t>
+          <t>LV</t>
         </is>
       </c>
       <c r="C3" t="n">
         <v>2</v>
       </c>
       <c r="D3" t="n">
-        <v>3400.9</v>
+        <v>3779.2</v>
       </c>
       <c r="E3" t="n">
-        <v>1792.6</v>
+        <v>2870.1</v>
       </c>
       <c r="F3" t="n">
-        <v>16.16</v>
+        <v>17.12</v>
       </c>
       <c r="G3" t="n">
-        <v>8.529999999999999</v>
+        <v>13.07</v>
       </c>
       <c r="H3" t="n">
-        <v>282.1</v>
+        <v>223.3</v>
       </c>
       <c r="I3" t="n">
-        <v>150.4</v>
+        <v>171.1</v>
       </c>
       <c r="J3" t="n">
-        <v>2.89</v>
+        <v>3.89</v>
       </c>
       <c r="K3" t="n">
-        <v>1.56</v>
+        <v>2.94</v>
       </c>
       <c r="L3" t="n">
-        <v>12.11</v>
+        <v>12.73</v>
       </c>
       <c r="M3" t="n">
-        <v>6.4</v>
+        <v>9.73</v>
       </c>
       <c r="N3" t="n">
-        <v>4.97</v>
+        <v>2.72</v>
       </c>
       <c r="O3" t="n">
-        <v>2.65</v>
+        <v>2.07</v>
       </c>
       <c r="P3" t="n">
-        <v>212.07</v>
+        <v>234.42</v>
       </c>
       <c r="Q3" t="n">
-        <v>112.12</v>
+        <v>178.23</v>
       </c>
       <c r="R3" t="n">
-        <v>63.43</v>
+        <v>108.07</v>
       </c>
       <c r="S3" t="n">
-        <v>160.74</v>
+        <v>247.88</v>
       </c>
       <c r="T3" t="n">
-        <v>92.91</v>
+        <v>170.12</v>
       </c>
       <c r="U3" t="n">
-        <v>19.21</v>
-      </c>
-      <c r="V3" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
+        <v>8.109999999999999</v>
+      </c>
+      <c r="V3" t="inlineStr"/>
       <c r="W3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Jameis Winston</t>
+          <t>Shedeur Sanders</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>NYG</t>
+          <t>CLE</t>
         </is>
       </c>
       <c r="C4" t="n">
         <v>2</v>
       </c>
       <c r="D4" t="n">
-        <v>3385.3</v>
+        <v>3400.9</v>
       </c>
       <c r="E4" t="n">
-        <v>997.2</v>
+        <v>1792.6</v>
       </c>
       <c r="F4" t="n">
-        <v>23.03</v>
+        <v>16.16</v>
       </c>
       <c r="G4" t="n">
-        <v>6.88</v>
+        <v>8.529999999999999</v>
       </c>
       <c r="H4" t="n">
-        <v>188.9</v>
+        <v>282.1</v>
       </c>
       <c r="I4" t="n">
-        <v>55.3</v>
+        <v>150.4</v>
       </c>
       <c r="J4" t="n">
-        <v>2.33</v>
+        <v>2.89</v>
       </c>
       <c r="K4" t="n">
-        <v>0.6899999999999999</v>
+        <v>1.56</v>
       </c>
       <c r="L4" t="n">
-        <v>15.13</v>
+        <v>12.11</v>
       </c>
       <c r="M4" t="n">
-        <v>4.46</v>
+        <v>6.4</v>
       </c>
       <c r="N4" t="n">
-        <v>3.4</v>
+        <v>4.97</v>
       </c>
       <c r="O4" t="n">
-        <v>1</v>
+        <v>2.65</v>
       </c>
       <c r="P4" t="n">
-        <v>223.34</v>
+        <v>212.07</v>
       </c>
       <c r="Q4" t="n">
-        <v>66.16</v>
+        <v>112.12</v>
       </c>
       <c r="R4" t="n">
-        <v>39.28</v>
+        <v>63.43</v>
       </c>
       <c r="S4" t="n">
-        <v>93.44</v>
-      </c>
-      <c r="T4" t="inlineStr"/>
-      <c r="U4" t="inlineStr"/>
-      <c r="V4" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
+        <v>160.74</v>
+      </c>
+      <c r="T4" t="n">
+        <v>92.91</v>
+      </c>
+      <c r="U4" t="n">
+        <v>19.21</v>
+      </c>
+      <c r="V4" t="inlineStr"/>
       <c r="W4" t="inlineStr"/>
     </row>
     <row r="5">
@@ -8155,11 +7775,7 @@
       </c>
       <c r="T5" t="inlineStr"/>
       <c r="U5" t="inlineStr"/>
-      <c r="V5" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
+      <c r="V5" t="inlineStr"/>
       <c r="W5" t="inlineStr"/>
     </row>
     <row r="6">
@@ -8226,11 +7842,7 @@
       </c>
       <c r="T6" t="inlineStr"/>
       <c r="U6" t="inlineStr"/>
-      <c r="V6" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
+      <c r="V6" t="inlineStr"/>
       <c r="W6" t="inlineStr"/>
     </row>
     <row r="7">
@@ -8297,11 +7909,7 @@
       </c>
       <c r="T7" t="inlineStr"/>
       <c r="U7" t="inlineStr"/>
-      <c r="V7" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
+      <c r="V7" t="inlineStr"/>
       <c r="W7" t="inlineStr"/>
     </row>
     <row r="8">
@@ -8372,11 +7980,7 @@
       <c r="U8" t="n">
         <v>-21.18</v>
       </c>
-      <c r="V8" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
+      <c r="V8" t="inlineStr"/>
       <c r="W8" t="inlineStr"/>
     </row>
     <row r="9">
@@ -8510,11 +8114,7 @@
       </c>
       <c r="T10" t="inlineStr"/>
       <c r="U10" t="inlineStr"/>
-      <c r="V10" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
+      <c r="V10" t="inlineStr"/>
       <c r="W10" t="inlineStr"/>
     </row>
     <row r="11">
@@ -8581,11 +8181,7 @@
       </c>
       <c r="T11" t="inlineStr"/>
       <c r="U11" t="inlineStr"/>
-      <c r="V11" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
+      <c r="V11" t="inlineStr"/>
       <c r="W11" t="inlineStr"/>
     </row>
     <row r="12">
@@ -8652,11 +8248,7 @@
       </c>
       <c r="T12" t="inlineStr"/>
       <c r="U12" t="inlineStr"/>
-      <c r="V12" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
+      <c r="V12" t="inlineStr"/>
       <c r="W12" t="inlineStr"/>
     </row>
     <row r="13">
@@ -8790,11 +8382,7 @@
       </c>
       <c r="T14" t="inlineStr"/>
       <c r="U14" t="inlineStr"/>
-      <c r="V14" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
+      <c r="V14" t="inlineStr"/>
       <c r="W14" t="inlineStr"/>
     </row>
     <row r="15">
@@ -8861,11 +8449,7 @@
       </c>
       <c r="T15" t="inlineStr"/>
       <c r="U15" t="inlineStr"/>
-      <c r="V15" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
+      <c r="V15" t="inlineStr"/>
       <c r="W15" t="inlineStr"/>
     </row>
     <row r="16">
@@ -8999,11 +8583,7 @@
       </c>
       <c r="T17" t="inlineStr"/>
       <c r="U17" t="inlineStr"/>
-      <c r="V17" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
+      <c r="V17" t="inlineStr"/>
       <c r="W17" t="inlineStr"/>
     </row>
     <row r="18">
@@ -9070,11 +8650,7 @@
       </c>
       <c r="T18" t="inlineStr"/>
       <c r="U18" t="inlineStr"/>
-      <c r="V18" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
+      <c r="V18" t="inlineStr"/>
       <c r="W18" t="inlineStr"/>
     </row>
     <row r="19">
@@ -9141,11 +8717,7 @@
       </c>
       <c r="T19" t="inlineStr"/>
       <c r="U19" t="inlineStr"/>
-      <c r="V19" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
+      <c r="V19" t="inlineStr"/>
       <c r="W19" t="inlineStr"/>
     </row>
     <row r="20">
@@ -9279,11 +8851,7 @@
       </c>
       <c r="T21" t="inlineStr"/>
       <c r="U21" t="inlineStr"/>
-      <c r="V21" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
+      <c r="V21" t="inlineStr"/>
       <c r="W21" t="inlineStr"/>
     </row>
     <row r="22">
@@ -9350,11 +8918,7 @@
       </c>
       <c r="T22" t="inlineStr"/>
       <c r="U22" t="inlineStr"/>
-      <c r="V22" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
+      <c r="V22" t="inlineStr"/>
       <c r="W22" t="inlineStr"/>
     </row>
     <row r="23">
@@ -9421,11 +8985,7 @@
       </c>
       <c r="T23" t="inlineStr"/>
       <c r="U23" t="inlineStr"/>
-      <c r="V23" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
+      <c r="V23" t="inlineStr"/>
       <c r="W23" t="inlineStr"/>
     </row>
     <row r="24">
@@ -9492,11 +9052,7 @@
       </c>
       <c r="T24" t="inlineStr"/>
       <c r="U24" t="inlineStr"/>
-      <c r="V24" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
+      <c r="V24" t="inlineStr"/>
       <c r="W24" t="inlineStr"/>
     </row>
     <row r="25">
@@ -9630,11 +9186,7 @@
       </c>
       <c r="T26" t="inlineStr"/>
       <c r="U26" t="inlineStr"/>
-      <c r="V26" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
+      <c r="V26" t="inlineStr"/>
       <c r="W26" t="inlineStr"/>
     </row>
     <row r="27">
@@ -9768,11 +9320,7 @@
       </c>
       <c r="T28" t="inlineStr"/>
       <c r="U28" t="inlineStr"/>
-      <c r="V28" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
+      <c r="V28" t="inlineStr"/>
       <c r="W28" t="inlineStr"/>
     </row>
     <row r="29">
@@ -9839,11 +9387,7 @@
       </c>
       <c r="T29" t="inlineStr"/>
       <c r="U29" t="inlineStr"/>
-      <c r="V29" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
+      <c r="V29" t="inlineStr"/>
       <c r="W29" t="inlineStr"/>
     </row>
     <row r="30">
@@ -9914,11 +9458,7 @@
       <c r="U30" t="n">
         <v>-71.12</v>
       </c>
-      <c r="V30" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
+      <c r="V30" t="inlineStr"/>
       <c r="W30" t="inlineStr"/>
     </row>
     <row r="31">
@@ -9985,11 +9525,7 @@
       </c>
       <c r="T31" t="inlineStr"/>
       <c r="U31" t="inlineStr"/>
-      <c r="V31" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
+      <c r="V31" t="inlineStr"/>
       <c r="W31" t="inlineStr"/>
     </row>
     <row r="32">
@@ -10056,11 +9592,7 @@
       </c>
       <c r="T32" t="inlineStr"/>
       <c r="U32" t="inlineStr"/>
-      <c r="V32" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
+      <c r="V32" t="inlineStr"/>
       <c r="W32" t="inlineStr"/>
     </row>
     <row r="33">
@@ -10127,11 +9659,7 @@
       </c>
       <c r="T33" t="inlineStr"/>
       <c r="U33" t="inlineStr"/>
-      <c r="V33" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
+      <c r="V33" t="inlineStr"/>
       <c r="W33" t="inlineStr"/>
     </row>
   </sheetData>
@@ -32644,67 +32172,67 @@
         <v>0</v>
       </c>
       <c r="H242" t="n">
-        <v>0</v>
+        <v>213.72</v>
       </c>
       <c r="I242" t="n">
-        <v>0</v>
+        <v>1.438</v>
       </c>
       <c r="J242" t="n">
-        <v>0</v>
+        <v>42.393</v>
       </c>
       <c r="K242" t="n">
-        <v>0</v>
+        <v>0.445</v>
       </c>
       <c r="L242" t="n">
-        <v>0</v>
+        <v>0.604</v>
       </c>
       <c r="M242" t="n">
-        <v>0</v>
+        <v>0.235</v>
       </c>
       <c r="N242" t="n">
-        <v>0</v>
+        <v>120.597</v>
       </c>
       <c r="O242" t="n">
-        <v>0</v>
+        <v>306.843</v>
       </c>
       <c r="P242" t="n">
-        <v>0</v>
+        <v>0.498</v>
       </c>
       <c r="Q242" t="n">
-        <v>0</v>
+        <v>2.843</v>
       </c>
       <c r="R242" t="n">
-        <v>0</v>
+        <v>21.402</v>
       </c>
       <c r="S242" t="n">
-        <v>0</v>
+        <v>63.38</v>
       </c>
       <c r="T242" t="n">
-        <v>0</v>
+        <v>0.154</v>
       </c>
       <c r="U242" t="n">
-        <v>0</v>
+        <v>0.963</v>
       </c>
       <c r="V242" t="n">
-        <v>0</v>
+        <v>0.209</v>
       </c>
       <c r="W242" t="n">
-        <v>0</v>
+        <v>1.739</v>
       </c>
       <c r="X242" t="n">
-        <v>0</v>
+        <v>0.081</v>
       </c>
       <c r="Y242" t="n">
-        <v>0</v>
+        <v>0.832</v>
       </c>
       <c r="Z242" t="n">
-        <v>0</v>
+        <v>19.534</v>
       </c>
       <c r="AA242" t="n">
-        <v>0</v>
+        <v>4.738</v>
       </c>
       <c r="AB242" t="n">
-        <v>0</v>
+        <v>35.182</v>
       </c>
       <c r="AC242" t="inlineStr"/>
     </row>
@@ -33109,67 +32637,67 @@
         <v>0</v>
       </c>
       <c r="H247" t="n">
-        <v>205.022</v>
+        <v>0</v>
       </c>
       <c r="I247" t="n">
-        <v>1.315</v>
+        <v>0</v>
       </c>
       <c r="J247" t="n">
-        <v>42.18</v>
+        <v>0</v>
       </c>
       <c r="K247" t="n">
-        <v>0.445</v>
+        <v>0</v>
       </c>
       <c r="L247" t="n">
-        <v>0.601</v>
+        <v>0</v>
       </c>
       <c r="M247" t="n">
-        <v>0.235</v>
+        <v>0</v>
       </c>
       <c r="N247" t="n">
-        <v>111.904</v>
+        <v>0</v>
       </c>
       <c r="O247" t="n">
-        <v>298.144</v>
+        <v>0</v>
       </c>
       <c r="P247" t="n">
-        <v>0.455</v>
+        <v>0</v>
       </c>
       <c r="Q247" t="n">
-        <v>2.72</v>
+        <v>0</v>
       </c>
       <c r="R247" t="n">
-        <v>21.191</v>
+        <v>0</v>
       </c>
       <c r="S247" t="n">
-        <v>63.169</v>
+        <v>0</v>
       </c>
       <c r="T247" t="n">
-        <v>0.154</v>
+        <v>0</v>
       </c>
       <c r="U247" t="n">
-        <v>0.964</v>
+        <v>0</v>
       </c>
       <c r="V247" t="n">
-        <v>0.208</v>
+        <v>0</v>
       </c>
       <c r="W247" t="n">
-        <v>1.737</v>
+        <v>0</v>
       </c>
       <c r="X247" t="n">
-        <v>0.081</v>
+        <v>0</v>
       </c>
       <c r="Y247" t="n">
-        <v>0.832</v>
+        <v>0</v>
       </c>
       <c r="Z247" t="n">
-        <v>18.681</v>
+        <v>0</v>
       </c>
       <c r="AA247" t="n">
-        <v>4.204</v>
+        <v>0</v>
       </c>
       <c r="AB247" t="n">
-        <v>34.327</v>
+        <v>0</v>
       </c>
       <c r="AC247" t="inlineStr"/>
     </row>
@@ -33202,67 +32730,67 @@
         <v>0</v>
       </c>
       <c r="H248" t="n">
-        <v>209.761</v>
+        <v>0</v>
       </c>
       <c r="I248" t="n">
-        <v>1.444</v>
+        <v>0</v>
       </c>
       <c r="J248" t="n">
-        <v>42.628</v>
+        <v>0</v>
       </c>
       <c r="K248" t="n">
-        <v>0.471</v>
+        <v>0</v>
       </c>
       <c r="L248" t="n">
-        <v>0.602</v>
+        <v>0</v>
       </c>
       <c r="M248" t="n">
-        <v>0.235</v>
+        <v>0</v>
       </c>
       <c r="N248" t="n">
-        <v>116.637</v>
+        <v>0</v>
       </c>
       <c r="O248" t="n">
-        <v>302.884</v>
+        <v>0</v>
       </c>
       <c r="P248" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="Q248" t="n">
-        <v>2.849</v>
+        <v>0</v>
       </c>
       <c r="R248" t="n">
-        <v>21.64</v>
+        <v>0</v>
       </c>
       <c r="S248" t="n">
-        <v>63.618</v>
+        <v>0</v>
       </c>
       <c r="T248" t="n">
-        <v>0.163</v>
+        <v>0</v>
       </c>
       <c r="U248" t="n">
-        <v>0.989</v>
+        <v>0</v>
       </c>
       <c r="V248" t="n">
-        <v>0.209</v>
+        <v>0</v>
       </c>
       <c r="W248" t="n">
-        <v>1.738</v>
+        <v>0</v>
       </c>
       <c r="X248" t="n">
-        <v>0.081</v>
+        <v>0</v>
       </c>
       <c r="Y248" t="n">
-        <v>0.832</v>
+        <v>0</v>
       </c>
       <c r="Z248" t="n">
-        <v>19.58</v>
+        <v>0</v>
       </c>
       <c r="AA248" t="n">
-        <v>4.667</v>
+        <v>0</v>
       </c>
       <c r="AB248" t="n">
-        <v>35.227</v>
+        <v>0</v>
       </c>
       <c r="AC248" t="inlineStr"/>
     </row>
@@ -33295,67 +32823,67 @@
         <v>0</v>
       </c>
       <c r="H249" t="n">
-        <v>212.781</v>
+        <v>0</v>
       </c>
       <c r="I249" t="n">
-        <v>1.241</v>
+        <v>0</v>
       </c>
       <c r="J249" t="n">
-        <v>42.619</v>
+        <v>0</v>
       </c>
       <c r="K249" t="n">
-        <v>0.469</v>
+        <v>0</v>
       </c>
       <c r="L249" t="n">
-        <v>0.604</v>
+        <v>0</v>
       </c>
       <c r="M249" t="n">
-        <v>0.235</v>
+        <v>0</v>
       </c>
       <c r="N249" t="n">
-        <v>119.657</v>
+        <v>0</v>
       </c>
       <c r="O249" t="n">
-        <v>305.904</v>
+        <v>0</v>
       </c>
       <c r="P249" t="n">
-        <v>0.429</v>
+        <v>0</v>
       </c>
       <c r="Q249" t="n">
-        <v>2.645</v>
+        <v>0</v>
       </c>
       <c r="R249" t="n">
-        <v>21.631</v>
+        <v>0</v>
       </c>
       <c r="S249" t="n">
-        <v>63.609</v>
+        <v>0</v>
       </c>
       <c r="T249" t="n">
-        <v>0.162</v>
+        <v>0</v>
       </c>
       <c r="U249" t="n">
-        <v>0.987</v>
+        <v>0</v>
       </c>
       <c r="V249" t="n">
-        <v>0.209</v>
+        <v>0</v>
       </c>
       <c r="W249" t="n">
-        <v>1.74</v>
+        <v>0</v>
       </c>
       <c r="X249" t="n">
-        <v>0.081</v>
+        <v>0</v>
       </c>
       <c r="Y249" t="n">
-        <v>0.832</v>
+        <v>0</v>
       </c>
       <c r="Z249" t="n">
-        <v>18.872</v>
+        <v>0</v>
       </c>
       <c r="AA249" t="n">
-        <v>4.497</v>
+        <v>0</v>
       </c>
       <c r="AB249" t="n">
-        <v>34.519</v>
+        <v>0</v>
       </c>
       <c r="AC249" t="inlineStr"/>
     </row>
@@ -33388,67 +32916,67 @@
         <v>1</v>
       </c>
       <c r="H250" t="n">
-        <v>216.434</v>
+        <v>0</v>
       </c>
       <c r="I250" t="n">
-        <v>1.336</v>
+        <v>0</v>
       </c>
       <c r="J250" t="n">
-        <v>42.172</v>
+        <v>0</v>
       </c>
       <c r="K250" t="n">
-        <v>0.458</v>
+        <v>0</v>
       </c>
       <c r="L250" t="n">
-        <v>0.608</v>
+        <v>0</v>
       </c>
       <c r="M250" t="n">
-        <v>0.258</v>
+        <v>0</v>
       </c>
       <c r="N250" t="n">
-        <v>123.314</v>
+        <v>0</v>
       </c>
       <c r="O250" t="n">
-        <v>309.555</v>
+        <v>0</v>
       </c>
       <c r="P250" t="n">
-        <v>0.463</v>
+        <v>0</v>
       </c>
       <c r="Q250" t="n">
-        <v>2.741</v>
+        <v>0</v>
       </c>
       <c r="R250" t="n">
-        <v>21.182</v>
+        <v>0</v>
       </c>
       <c r="S250" t="n">
-        <v>63.16</v>
+        <v>0</v>
       </c>
       <c r="T250" t="n">
-        <v>0.159</v>
+        <v>0</v>
       </c>
       <c r="U250" t="n">
-        <v>0.977</v>
+        <v>0</v>
       </c>
       <c r="V250" t="n">
-        <v>0.211</v>
+        <v>0</v>
       </c>
       <c r="W250" t="n">
-        <v>1.744</v>
+        <v>0</v>
       </c>
       <c r="X250" t="n">
-        <v>0.089</v>
+        <v>0</v>
       </c>
       <c r="Y250" t="n">
-        <v>0.855</v>
+        <v>0</v>
       </c>
       <c r="Z250" t="n">
-        <v>19.238</v>
+        <v>0</v>
       </c>
       <c r="AA250" t="n">
-        <v>4.656</v>
+        <v>0</v>
       </c>
       <c r="AB250" t="n">
-        <v>34.924</v>
+        <v>0</v>
       </c>
       <c r="AC250" t="inlineStr"/>
     </row>
@@ -33481,67 +33009,67 @@
         <v>0</v>
       </c>
       <c r="H251" t="n">
-        <v>214.566</v>
+        <v>0</v>
       </c>
       <c r="I251" t="n">
-        <v>1.337</v>
+        <v>0</v>
       </c>
       <c r="J251" t="n">
-        <v>42.601</v>
+        <v>0</v>
       </c>
       <c r="K251" t="n">
-        <v>0.475</v>
+        <v>0</v>
       </c>
       <c r="L251" t="n">
-        <v>0.603</v>
+        <v>0</v>
       </c>
       <c r="M251" t="n">
-        <v>0.235</v>
+        <v>0</v>
       </c>
       <c r="N251" t="n">
-        <v>121.445</v>
+        <v>0</v>
       </c>
       <c r="O251" t="n">
-        <v>307.686</v>
+        <v>0</v>
       </c>
       <c r="P251" t="n">
-        <v>0.463</v>
+        <v>0</v>
       </c>
       <c r="Q251" t="n">
-        <v>2.741</v>
+        <v>0</v>
       </c>
       <c r="R251" t="n">
-        <v>21.611</v>
+        <v>0</v>
       </c>
       <c r="S251" t="n">
-        <v>63.589</v>
+        <v>0</v>
       </c>
       <c r="T251" t="n">
-        <v>0.165</v>
+        <v>0</v>
       </c>
       <c r="U251" t="n">
-        <v>0.994</v>
+        <v>0</v>
       </c>
       <c r="V251" t="n">
-        <v>0.209</v>
+        <v>0</v>
       </c>
       <c r="W251" t="n">
-        <v>1.739</v>
+        <v>0</v>
       </c>
       <c r="X251" t="n">
-        <v>0.081</v>
+        <v>0</v>
       </c>
       <c r="Y251" t="n">
-        <v>0.832</v>
+        <v>0</v>
       </c>
       <c r="Z251" t="n">
-        <v>19.367</v>
+        <v>0</v>
       </c>
       <c r="AA251" t="n">
-        <v>4.716</v>
+        <v>0</v>
       </c>
       <c r="AB251" t="n">
-        <v>35.014</v>
+        <v>0</v>
       </c>
       <c r="AC251" t="inlineStr"/>
     </row>
@@ -33574,67 +33102,67 @@
         <v>0</v>
       </c>
       <c r="H252" t="n">
-        <v>210.139</v>
+        <v>0</v>
       </c>
       <c r="I252" t="n">
-        <v>1.254</v>
+        <v>0</v>
       </c>
       <c r="J252" t="n">
-        <v>42.275</v>
+        <v>0</v>
       </c>
       <c r="K252" t="n">
-        <v>0.448</v>
+        <v>0</v>
       </c>
       <c r="L252" t="n">
-        <v>0.605</v>
+        <v>0</v>
       </c>
       <c r="M252" t="n">
-        <v>0.235</v>
+        <v>0</v>
       </c>
       <c r="N252" t="n">
-        <v>117.016</v>
+        <v>0</v>
       </c>
       <c r="O252" t="n">
-        <v>303.263</v>
+        <v>0</v>
       </c>
       <c r="P252" t="n">
-        <v>0.434</v>
+        <v>0</v>
       </c>
       <c r="Q252" t="n">
-        <v>2.659</v>
+        <v>0</v>
       </c>
       <c r="R252" t="n">
-        <v>21.283</v>
+        <v>0</v>
       </c>
       <c r="S252" t="n">
-        <v>63.267</v>
+        <v>0</v>
       </c>
       <c r="T252" t="n">
-        <v>0.155</v>
+        <v>0</v>
       </c>
       <c r="U252" t="n">
-        <v>0.966</v>
+        <v>0</v>
       </c>
       <c r="V252" t="n">
-        <v>0.209</v>
+        <v>0</v>
       </c>
       <c r="W252" t="n">
-        <v>1.741</v>
+        <v>0</v>
       </c>
       <c r="X252" t="n">
-        <v>0.081</v>
+        <v>0</v>
       </c>
       <c r="Y252" t="n">
-        <v>0.832</v>
+        <v>0</v>
       </c>
       <c r="Z252" t="n">
-        <v>18.656</v>
+        <v>0</v>
       </c>
       <c r="AA252" t="n">
-        <v>4.33</v>
+        <v>0</v>
       </c>
       <c r="AB252" t="n">
-        <v>34.304</v>
+        <v>0</v>
       </c>
       <c r="AC252" t="inlineStr"/>
     </row>
@@ -33667,67 +33195,67 @@
         <v>0</v>
       </c>
       <c r="H253" t="n">
-        <v>212.349</v>
+        <v>0</v>
       </c>
       <c r="I253" t="n">
-        <v>1.339</v>
+        <v>0</v>
       </c>
       <c r="J253" t="n">
-        <v>42.67</v>
+        <v>0</v>
       </c>
       <c r="K253" t="n">
-        <v>0.467</v>
+        <v>0</v>
       </c>
       <c r="L253" t="n">
-        <v>0.597</v>
+        <v>0</v>
       </c>
       <c r="M253" t="n">
-        <v>0.235</v>
+        <v>0</v>
       </c>
       <c r="N253" t="n">
-        <v>119.226</v>
+        <v>0</v>
       </c>
       <c r="O253" t="n">
-        <v>305.473</v>
+        <v>0</v>
       </c>
       <c r="P253" t="n">
-        <v>0.463</v>
+        <v>0</v>
       </c>
       <c r="Q253" t="n">
-        <v>2.743</v>
+        <v>0</v>
       </c>
       <c r="R253" t="n">
-        <v>21.681</v>
+        <v>0</v>
       </c>
       <c r="S253" t="n">
-        <v>63.659</v>
+        <v>0</v>
       </c>
       <c r="T253" t="n">
-        <v>0.162</v>
+        <v>0</v>
       </c>
       <c r="U253" t="n">
-        <v>0.985</v>
+        <v>0</v>
       </c>
       <c r="V253" t="n">
-        <v>0.207</v>
+        <v>0</v>
       </c>
       <c r="W253" t="n">
-        <v>1.733</v>
+        <v>0</v>
       </c>
       <c r="X253" t="n">
-        <v>0.081</v>
+        <v>0</v>
       </c>
       <c r="Y253" t="n">
-        <v>0.832</v>
+        <v>0</v>
       </c>
       <c r="Z253" t="n">
-        <v>19.251</v>
+        <v>0</v>
       </c>
       <c r="AA253" t="n">
-        <v>4.63</v>
+        <v>0</v>
       </c>
       <c r="AB253" t="n">
-        <v>34.891</v>
+        <v>0</v>
       </c>
       <c r="AC253" t="inlineStr"/>
     </row>
@@ -33760,67 +33288,67 @@
         <v>1</v>
       </c>
       <c r="H254" t="n">
-        <v>211.606</v>
+        <v>0</v>
       </c>
       <c r="I254" t="n">
-        <v>1.341</v>
+        <v>0</v>
       </c>
       <c r="J254" t="n">
-        <v>42.122</v>
+        <v>0</v>
       </c>
       <c r="K254" t="n">
-        <v>0.433</v>
+        <v>0</v>
       </c>
       <c r="L254" t="n">
-        <v>0.602</v>
+        <v>0</v>
       </c>
       <c r="M254" t="n">
-        <v>0.258</v>
+        <v>0</v>
       </c>
       <c r="N254" t="n">
-        <v>118.485</v>
+        <v>0</v>
       </c>
       <c r="O254" t="n">
-        <v>304.726</v>
+        <v>0</v>
       </c>
       <c r="P254" t="n">
-        <v>0.464</v>
+        <v>0</v>
       </c>
       <c r="Q254" t="n">
-        <v>2.746</v>
+        <v>0</v>
       </c>
       <c r="R254" t="n">
-        <v>21.132</v>
+        <v>0</v>
       </c>
       <c r="S254" t="n">
-        <v>63.11</v>
+        <v>0</v>
       </c>
       <c r="T254" t="n">
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="U254" t="n">
-        <v>0.952</v>
+        <v>0</v>
       </c>
       <c r="V254" t="n">
-        <v>0.208</v>
+        <v>0</v>
       </c>
       <c r="W254" t="n">
-        <v>1.737</v>
+        <v>0</v>
       </c>
       <c r="X254" t="n">
-        <v>0.089</v>
+        <v>0</v>
       </c>
       <c r="Y254" t="n">
-        <v>0.855</v>
+        <v>0</v>
       </c>
       <c r="Z254" t="n">
-        <v>18.923</v>
+        <v>0</v>
       </c>
       <c r="AA254" t="n">
-        <v>4.426</v>
+        <v>0</v>
       </c>
       <c r="AB254" t="n">
-        <v>34.6</v>
+        <v>0</v>
       </c>
       <c r="AC254" t="inlineStr"/>
     </row>
@@ -33853,67 +33381,67 @@
         <v>1</v>
       </c>
       <c r="H255" t="n">
-        <v>218.992</v>
+        <v>0</v>
       </c>
       <c r="I255" t="n">
-        <v>1.446</v>
+        <v>0</v>
       </c>
       <c r="J255" t="n">
-        <v>42.138</v>
+        <v>0</v>
       </c>
       <c r="K255" t="n">
-        <v>0.432</v>
+        <v>0</v>
       </c>
       <c r="L255" t="n">
-        <v>0.598</v>
+        <v>0</v>
       </c>
       <c r="M255" t="n">
-        <v>0.258</v>
+        <v>0</v>
       </c>
       <c r="N255" t="n">
-        <v>125.874</v>
+        <v>0</v>
       </c>
       <c r="O255" t="n">
-        <v>312.114</v>
+        <v>0</v>
       </c>
       <c r="P255" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="Q255" t="n">
-        <v>2.85</v>
+        <v>0</v>
       </c>
       <c r="R255" t="n">
-        <v>21.15</v>
+        <v>0</v>
       </c>
       <c r="S255" t="n">
-        <v>63.128</v>
+        <v>0</v>
       </c>
       <c r="T255" t="n">
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="U255" t="n">
-        <v>0.951</v>
+        <v>0</v>
       </c>
       <c r="V255" t="n">
-        <v>0.207</v>
+        <v>0</v>
       </c>
       <c r="W255" t="n">
-        <v>1.733</v>
+        <v>0</v>
       </c>
       <c r="X255" t="n">
-        <v>0.089</v>
+        <v>0</v>
       </c>
       <c r="Y255" t="n">
-        <v>0.855</v>
+        <v>0</v>
       </c>
       <c r="Z255" t="n">
-        <v>19.641</v>
+        <v>0</v>
       </c>
       <c r="AA255" t="n">
-        <v>4.874</v>
+        <v>0</v>
       </c>
       <c r="AB255" t="n">
-        <v>35.311</v>
+        <v>0</v>
       </c>
       <c r="AC255" t="inlineStr"/>
     </row>
@@ -33946,67 +33474,67 @@
         <v>0</v>
       </c>
       <c r="H256" t="n">
-        <v>200.869</v>
+        <v>0</v>
       </c>
       <c r="I256" t="n">
-        <v>1.263</v>
+        <v>0</v>
       </c>
       <c r="J256" t="n">
-        <v>42.62</v>
+        <v>0</v>
       </c>
       <c r="K256" t="n">
-        <v>0.433</v>
+        <v>0</v>
       </c>
       <c r="L256" t="n">
-        <v>0.591</v>
+        <v>0</v>
       </c>
       <c r="M256" t="n">
-        <v>0.235</v>
+        <v>0</v>
       </c>
       <c r="N256" t="n">
-        <v>107.746</v>
+        <v>0</v>
       </c>
       <c r="O256" t="n">
-        <v>293.993</v>
+        <v>0</v>
       </c>
       <c r="P256" t="n">
-        <v>0.437</v>
+        <v>0</v>
       </c>
       <c r="Q256" t="n">
-        <v>2.668</v>
+        <v>0</v>
       </c>
       <c r="R256" t="n">
-        <v>21.631</v>
+        <v>0</v>
       </c>
       <c r="S256" t="n">
-        <v>63.609</v>
+        <v>0</v>
       </c>
       <c r="T256" t="n">
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="U256" t="n">
-        <v>0.951</v>
+        <v>0</v>
       </c>
       <c r="V256" t="n">
-        <v>0.205</v>
+        <v>0</v>
       </c>
       <c r="W256" t="n">
-        <v>1.727</v>
+        <v>0</v>
       </c>
       <c r="X256" t="n">
-        <v>0.081</v>
+        <v>0</v>
       </c>
       <c r="Y256" t="n">
-        <v>0.832</v>
+        <v>0</v>
       </c>
       <c r="Z256" t="n">
-        <v>18.293</v>
+        <v>0</v>
       </c>
       <c r="AA256" t="n">
-        <v>4.003</v>
+        <v>0</v>
       </c>
       <c r="AB256" t="n">
-        <v>33.924</v>
+        <v>0</v>
       </c>
       <c r="AC256" t="inlineStr"/>
     </row>
@@ -67519,67 +67047,67 @@
         <v>0</v>
       </c>
       <c r="H617" t="n">
-        <v>200.226</v>
+        <v>0</v>
       </c>
       <c r="I617" t="n">
-        <v>1.416</v>
+        <v>0</v>
       </c>
       <c r="J617" t="n">
-        <v>11.154</v>
+        <v>0</v>
       </c>
       <c r="K617" t="n">
-        <v>0.139</v>
+        <v>0</v>
       </c>
       <c r="L617" t="n">
-        <v>0.89</v>
+        <v>0</v>
       </c>
       <c r="M617" t="n">
-        <v>0.198</v>
+        <v>0</v>
       </c>
       <c r="N617" t="n">
-        <v>107.105</v>
+        <v>0</v>
       </c>
       <c r="O617" t="n">
-        <v>293.345</v>
+        <v>0</v>
       </c>
       <c r="P617" t="n">
-        <v>0.49</v>
+        <v>0</v>
       </c>
       <c r="Q617" t="n">
-        <v>2.82</v>
+        <v>0</v>
       </c>
       <c r="R617" t="n">
-        <v>3.861</v>
+        <v>0</v>
       </c>
       <c r="S617" t="n">
-        <v>32.147</v>
+        <v>0</v>
       </c>
       <c r="T617" t="n">
-        <v>0.048</v>
+        <v>0</v>
       </c>
       <c r="U617" t="n">
-        <v>0.657</v>
+        <v>0</v>
       </c>
       <c r="V617" t="n">
-        <v>0.308</v>
+        <v>0</v>
       </c>
       <c r="W617" t="n">
-        <v>2.026</v>
+        <v>0</v>
       </c>
       <c r="X617" t="n">
-        <v>0.06900000000000001</v>
+        <v>0</v>
       </c>
       <c r="Y617" t="n">
-        <v>0.796</v>
+        <v>0</v>
       </c>
       <c r="Z617" t="n">
-        <v>13.442</v>
+        <v>0</v>
       </c>
       <c r="AA617" t="n">
-        <v>1.275</v>
+        <v>0</v>
       </c>
       <c r="AB617" t="n">
-        <v>29.417</v>
+        <v>0</v>
       </c>
       <c r="AC617" t="inlineStr"/>
     </row>
@@ -67984,67 +67512,67 @@
         <v>0</v>
       </c>
       <c r="H622" t="n">
-        <v>0</v>
+        <v>191.528</v>
       </c>
       <c r="I622" t="n">
-        <v>0</v>
+        <v>1.317</v>
       </c>
       <c r="J622" t="n">
-        <v>0</v>
+        <v>10.941</v>
       </c>
       <c r="K622" t="n">
-        <v>0</v>
+        <v>0.139</v>
       </c>
       <c r="L622" t="n">
-        <v>0</v>
+        <v>0.888</v>
       </c>
       <c r="M622" t="n">
-        <v>0</v>
+        <v>0.198</v>
       </c>
       <c r="N622" t="n">
-        <v>0</v>
+        <v>98.40600000000001</v>
       </c>
       <c r="O622" t="n">
-        <v>0</v>
+        <v>284.646</v>
       </c>
       <c r="P622" t="n">
-        <v>0</v>
+        <v>0.456</v>
       </c>
       <c r="Q622" t="n">
-        <v>0</v>
+        <v>2.721</v>
       </c>
       <c r="R622" t="n">
-        <v>0</v>
+        <v>3.787</v>
       </c>
       <c r="S622" t="n">
-        <v>0</v>
+        <v>31.93</v>
       </c>
       <c r="T622" t="n">
-        <v>0</v>
+        <v>0.048</v>
       </c>
       <c r="U622" t="n">
-        <v>0</v>
+        <v>0.657</v>
       </c>
       <c r="V622" t="n">
-        <v>0</v>
+        <v>0.307</v>
       </c>
       <c r="W622" t="n">
-        <v>0</v>
+        <v>2.024</v>
       </c>
       <c r="X622" t="n">
-        <v>0</v>
+        <v>0.06900000000000001</v>
       </c>
       <c r="Y622" t="n">
-        <v>0</v>
+        <v>0.796</v>
       </c>
       <c r="Z622" t="n">
-        <v>0</v>
+        <v>12.682</v>
       </c>
       <c r="AA622" t="n">
-        <v>0</v>
+        <v>0.787</v>
       </c>
       <c r="AB622" t="n">
-        <v>0</v>
+        <v>28.653</v>
       </c>
       <c r="AC622" t="inlineStr"/>
     </row>
@@ -68077,67 +67605,67 @@
         <v>0</v>
       </c>
       <c r="H623" t="n">
-        <v>0</v>
+        <v>196.267</v>
       </c>
       <c r="I623" t="n">
-        <v>0</v>
+        <v>1.451</v>
       </c>
       <c r="J623" t="n">
-        <v>0</v>
+        <v>11.389</v>
       </c>
       <c r="K623" t="n">
-        <v>0</v>
+        <v>0.14</v>
       </c>
       <c r="L623" t="n">
-        <v>0</v>
+        <v>0.89</v>
       </c>
       <c r="M623" t="n">
-        <v>0</v>
+        <v>0.198</v>
       </c>
       <c r="N623" t="n">
-        <v>0</v>
+        <v>103.145</v>
       </c>
       <c r="O623" t="n">
-        <v>0</v>
+        <v>289.386</v>
       </c>
       <c r="P623" t="n">
-        <v>0</v>
+        <v>0.502</v>
       </c>
       <c r="Q623" t="n">
-        <v>0</v>
+        <v>2.856</v>
       </c>
       <c r="R623" t="n">
-        <v>0</v>
+        <v>3.942</v>
       </c>
       <c r="S623" t="n">
-        <v>0</v>
+        <v>32.379</v>
       </c>
       <c r="T623" t="n">
-        <v>0</v>
+        <v>0.048</v>
       </c>
       <c r="U623" t="n">
-        <v>0</v>
+        <v>0.658</v>
       </c>
       <c r="V623" t="n">
-        <v>0</v>
+        <v>0.308</v>
       </c>
       <c r="W623" t="n">
-        <v>0</v>
+        <v>2.026</v>
       </c>
       <c r="X623" t="n">
-        <v>0</v>
+        <v>0.06900000000000001</v>
       </c>
       <c r="Y623" t="n">
-        <v>0</v>
+        <v>0.796</v>
       </c>
       <c r="Z623" t="n">
-        <v>0</v>
+        <v>13.456</v>
       </c>
       <c r="AA623" t="n">
-        <v>0</v>
+        <v>1.176</v>
       </c>
       <c r="AB623" t="n">
-        <v>0</v>
+        <v>29.431</v>
       </c>
       <c r="AC623" t="inlineStr"/>
     </row>
@@ -68170,67 +67698,67 @@
         <v>0</v>
       </c>
       <c r="H624" t="n">
-        <v>0</v>
+        <v>199.287</v>
       </c>
       <c r="I624" t="n">
-        <v>0</v>
+        <v>1.238</v>
       </c>
       <c r="J624" t="n">
-        <v>0</v>
+        <v>11.38</v>
       </c>
       <c r="K624" t="n">
-        <v>0</v>
+        <v>0.136</v>
       </c>
       <c r="L624" t="n">
-        <v>0</v>
+        <v>0.892</v>
       </c>
       <c r="M624" t="n">
-        <v>0</v>
+        <v>0.198</v>
       </c>
       <c r="N624" t="n">
-        <v>0</v>
+        <v>106.165</v>
       </c>
       <c r="O624" t="n">
-        <v>0</v>
+        <v>292.406</v>
       </c>
       <c r="P624" t="n">
-        <v>0</v>
+        <v>0.429</v>
       </c>
       <c r="Q624" t="n">
-        <v>0</v>
+        <v>2.643</v>
       </c>
       <c r="R624" t="n">
-        <v>0</v>
+        <v>3.939</v>
       </c>
       <c r="S624" t="n">
-        <v>0</v>
+        <v>32.369</v>
       </c>
       <c r="T624" t="n">
-        <v>0</v>
+        <v>0.047</v>
       </c>
       <c r="U624" t="n">
-        <v>0</v>
+        <v>0.654</v>
       </c>
       <c r="V624" t="n">
-        <v>0</v>
+        <v>0.309</v>
       </c>
       <c r="W624" t="n">
-        <v>0</v>
+        <v>2.027</v>
       </c>
       <c r="X624" t="n">
-        <v>0</v>
+        <v>0.06900000000000001</v>
       </c>
       <c r="Y624" t="n">
-        <v>0</v>
+        <v>0.796</v>
       </c>
       <c r="Z624" t="n">
-        <v>0</v>
+        <v>12.699</v>
       </c>
       <c r="AA624" t="n">
-        <v>0</v>
+        <v>0.992</v>
       </c>
       <c r="AB624" t="n">
-        <v>0</v>
+        <v>28.675</v>
       </c>
       <c r="AC624" t="inlineStr"/>
     </row>
@@ -68263,67 +67791,67 @@
         <v>1</v>
       </c>
       <c r="H625" t="n">
-        <v>0</v>
+        <v>202.94</v>
       </c>
       <c r="I625" t="n">
-        <v>0</v>
+        <v>1.345</v>
       </c>
       <c r="J625" t="n">
-        <v>0</v>
+        <v>10.933</v>
       </c>
       <c r="K625" t="n">
-        <v>0</v>
+        <v>0.139</v>
       </c>
       <c r="L625" t="n">
-        <v>0</v>
+        <v>0.895</v>
       </c>
       <c r="M625" t="n">
-        <v>0</v>
+        <v>0.204</v>
       </c>
       <c r="N625" t="n">
-        <v>0</v>
+        <v>109.816</v>
       </c>
       <c r="O625" t="n">
-        <v>0</v>
+        <v>296.063</v>
       </c>
       <c r="P625" t="n">
-        <v>0</v>
+        <v>0.465</v>
       </c>
       <c r="Q625" t="n">
-        <v>0</v>
+        <v>2.749</v>
       </c>
       <c r="R625" t="n">
-        <v>0</v>
+        <v>3.784</v>
       </c>
       <c r="S625" t="n">
-        <v>0</v>
+        <v>31.92</v>
       </c>
       <c r="T625" t="n">
-        <v>0</v>
+        <v>0.048</v>
       </c>
       <c r="U625" t="n">
-        <v>0</v>
+        <v>0.658</v>
       </c>
       <c r="V625" t="n">
-        <v>0</v>
+        <v>0.31</v>
       </c>
       <c r="W625" t="n">
-        <v>0</v>
+        <v>2.031</v>
       </c>
       <c r="X625" t="n">
-        <v>0</v>
+        <v>0.07099999999999999</v>
       </c>
       <c r="Y625" t="n">
-        <v>0</v>
+        <v>0.802</v>
       </c>
       <c r="Z625" t="n">
-        <v>0</v>
+        <v>13.227</v>
       </c>
       <c r="AA625" t="n">
-        <v>0</v>
+        <v>1.257</v>
       </c>
       <c r="AB625" t="n">
-        <v>0</v>
+        <v>29.217</v>
       </c>
       <c r="AC625" t="inlineStr"/>
     </row>
@@ -68356,67 +67884,67 @@
         <v>0</v>
       </c>
       <c r="H626" t="n">
-        <v>0</v>
+        <v>201.072</v>
       </c>
       <c r="I626" t="n">
-        <v>0</v>
+        <v>1.343</v>
       </c>
       <c r="J626" t="n">
-        <v>0</v>
+        <v>11.362</v>
       </c>
       <c r="K626" t="n">
-        <v>0</v>
+        <v>0.136</v>
       </c>
       <c r="L626" t="n">
-        <v>0</v>
+        <v>0.891</v>
       </c>
       <c r="M626" t="n">
-        <v>0</v>
+        <v>0.198</v>
       </c>
       <c r="N626" t="n">
-        <v>0</v>
+        <v>107.954</v>
       </c>
       <c r="O626" t="n">
-        <v>0</v>
+        <v>294.194</v>
       </c>
       <c r="P626" t="n">
-        <v>0</v>
+        <v>0.465</v>
       </c>
       <c r="Q626" t="n">
-        <v>0</v>
+        <v>2.748</v>
       </c>
       <c r="R626" t="n">
-        <v>0</v>
+        <v>3.933</v>
       </c>
       <c r="S626" t="n">
-        <v>0</v>
+        <v>32.35</v>
       </c>
       <c r="T626" t="n">
-        <v>0</v>
+        <v>0.047</v>
       </c>
       <c r="U626" t="n">
-        <v>0</v>
+        <v>0.655</v>
       </c>
       <c r="V626" t="n">
-        <v>0</v>
+        <v>0.308</v>
       </c>
       <c r="W626" t="n">
-        <v>0</v>
+        <v>2.027</v>
       </c>
       <c r="X626" t="n">
-        <v>0</v>
+        <v>0.06900000000000001</v>
       </c>
       <c r="Y626" t="n">
-        <v>0</v>
+        <v>0.796</v>
       </c>
       <c r="Z626" t="n">
-        <v>0</v>
+        <v>13.193</v>
       </c>
       <c r="AA626" t="n">
-        <v>0</v>
+        <v>1.21</v>
       </c>
       <c r="AB626" t="n">
-        <v>0</v>
+        <v>29.17</v>
       </c>
       <c r="AC626" t="inlineStr"/>
     </row>
@@ -68449,67 +67977,67 @@
         <v>0</v>
       </c>
       <c r="H627" t="n">
-        <v>0</v>
+        <v>196.645</v>
       </c>
       <c r="I627" t="n">
-        <v>0</v>
+        <v>1.262</v>
       </c>
       <c r="J627" t="n">
-        <v>0</v>
+        <v>11.036</v>
       </c>
       <c r="K627" t="n">
-        <v>0</v>
+        <v>0.135</v>
       </c>
       <c r="L627" t="n">
-        <v>0</v>
+        <v>0.893</v>
       </c>
       <c r="M627" t="n">
-        <v>0</v>
+        <v>0.198</v>
       </c>
       <c r="N627" t="n">
-        <v>0</v>
+        <v>103.525</v>
       </c>
       <c r="O627" t="n">
-        <v>0</v>
+        <v>289.765</v>
       </c>
       <c r="P627" t="n">
-        <v>0</v>
+        <v>0.437</v>
       </c>
       <c r="Q627" t="n">
-        <v>0</v>
+        <v>2.666</v>
       </c>
       <c r="R627" t="n">
-        <v>0</v>
+        <v>3.82</v>
       </c>
       <c r="S627" t="n">
-        <v>0</v>
+        <v>32.028</v>
       </c>
       <c r="T627" t="n">
-        <v>0</v>
+        <v>0.047</v>
       </c>
       <c r="U627" t="n">
-        <v>0</v>
+        <v>0.653</v>
       </c>
       <c r="V627" t="n">
-        <v>0</v>
+        <v>0.309</v>
       </c>
       <c r="W627" t="n">
-        <v>0</v>
+        <v>2.028</v>
       </c>
       <c r="X627" t="n">
-        <v>0</v>
+        <v>0.06900000000000001</v>
       </c>
       <c r="Y627" t="n">
-        <v>0</v>
+        <v>0.796</v>
       </c>
       <c r="Z627" t="n">
-        <v>0</v>
+        <v>12.643</v>
       </c>
       <c r="AA627" t="n">
-        <v>0</v>
+        <v>0.902</v>
       </c>
       <c r="AB627" t="n">
-        <v>0</v>
+        <v>28.62</v>
       </c>
       <c r="AC627" t="inlineStr"/>
     </row>
@@ -68542,67 +68070,67 @@
         <v>0</v>
       </c>
       <c r="H628" t="n">
-        <v>0</v>
+        <v>198.855</v>
       </c>
       <c r="I628" t="n">
-        <v>0</v>
+        <v>1.331</v>
       </c>
       <c r="J628" t="n">
-        <v>0</v>
+        <v>11.431</v>
       </c>
       <c r="K628" t="n">
-        <v>0</v>
+        <v>0.143</v>
       </c>
       <c r="L628" t="n">
-        <v>0</v>
+        <v>0.886</v>
       </c>
       <c r="M628" t="n">
-        <v>0</v>
+        <v>0.198</v>
       </c>
       <c r="N628" t="n">
-        <v>0</v>
+        <v>105.735</v>
       </c>
       <c r="O628" t="n">
-        <v>0</v>
+        <v>291.975</v>
       </c>
       <c r="P628" t="n">
-        <v>0</v>
+        <v>0.461</v>
       </c>
       <c r="Q628" t="n">
-        <v>0</v>
+        <v>2.736</v>
       </c>
       <c r="R628" t="n">
-        <v>0</v>
+        <v>3.957</v>
       </c>
       <c r="S628" t="n">
-        <v>0</v>
+        <v>32.42</v>
       </c>
       <c r="T628" t="n">
-        <v>0</v>
+        <v>0.049</v>
       </c>
       <c r="U628" t="n">
-        <v>0</v>
+        <v>0.661</v>
       </c>
       <c r="V628" t="n">
-        <v>0</v>
+        <v>0.307</v>
       </c>
       <c r="W628" t="n">
-        <v>0</v>
+        <v>2.021</v>
       </c>
       <c r="X628" t="n">
-        <v>0</v>
+        <v>0.06900000000000001</v>
       </c>
       <c r="Y628" t="n">
-        <v>0</v>
+        <v>0.796</v>
       </c>
       <c r="Z628" t="n">
-        <v>0</v>
+        <v>13.109</v>
       </c>
       <c r="AA628" t="n">
-        <v>0</v>
+        <v>1.131</v>
       </c>
       <c r="AB628" t="n">
-        <v>0</v>
+        <v>29.077</v>
       </c>
       <c r="AC628" t="inlineStr"/>
     </row>
@@ -68635,67 +68163,67 @@
         <v>1</v>
       </c>
       <c r="H629" t="n">
-        <v>0</v>
+        <v>198.112</v>
       </c>
       <c r="I629" t="n">
-        <v>0</v>
+        <v>1.347</v>
       </c>
       <c r="J629" t="n">
-        <v>0</v>
+        <v>10.883</v>
       </c>
       <c r="K629" t="n">
-        <v>0</v>
+        <v>0.136</v>
       </c>
       <c r="L629" t="n">
-        <v>0</v>
+        <v>0.889</v>
       </c>
       <c r="M629" t="n">
-        <v>0</v>
+        <v>0.204</v>
       </c>
       <c r="N629" t="n">
-        <v>0</v>
+        <v>104.994</v>
       </c>
       <c r="O629" t="n">
-        <v>0</v>
+        <v>291.234</v>
       </c>
       <c r="P629" t="n">
-        <v>0</v>
+        <v>0.466</v>
       </c>
       <c r="Q629" t="n">
-        <v>0</v>
+        <v>2.752</v>
       </c>
       <c r="R629" t="n">
-        <v>0</v>
+        <v>3.767</v>
       </c>
       <c r="S629" t="n">
-        <v>0</v>
+        <v>31.87</v>
       </c>
       <c r="T629" t="n">
-        <v>0</v>
+        <v>0.047</v>
       </c>
       <c r="U629" t="n">
-        <v>0</v>
+        <v>0.654</v>
       </c>
       <c r="V629" t="n">
-        <v>0</v>
+        <v>0.308</v>
       </c>
       <c r="W629" t="n">
-        <v>0</v>
+        <v>2.025</v>
       </c>
       <c r="X629" t="n">
-        <v>0</v>
+        <v>0.07099999999999999</v>
       </c>
       <c r="Y629" t="n">
-        <v>0</v>
+        <v>0.802</v>
       </c>
       <c r="Z629" t="n">
-        <v>0</v>
+        <v>13.027</v>
       </c>
       <c r="AA629" t="n">
-        <v>0</v>
+        <v>1.07</v>
       </c>
       <c r="AB629" t="n">
-        <v>0</v>
+        <v>29.007</v>
       </c>
       <c r="AC629" t="inlineStr"/>
     </row>
@@ -68728,67 +68256,67 @@
         <v>1</v>
       </c>
       <c r="H630" t="n">
-        <v>0</v>
+        <v>205.498</v>
       </c>
       <c r="I630" t="n">
-        <v>0</v>
+        <v>1.436</v>
       </c>
       <c r="J630" t="n">
-        <v>0</v>
+        <v>10.899</v>
       </c>
       <c r="K630" t="n">
-        <v>0</v>
+        <v>0.137</v>
       </c>
       <c r="L630" t="n">
-        <v>0</v>
+        <v>0.885</v>
       </c>
       <c r="M630" t="n">
-        <v>0</v>
+        <v>0.204</v>
       </c>
       <c r="N630" t="n">
-        <v>0</v>
+        <v>112.376</v>
       </c>
       <c r="O630" t="n">
-        <v>0</v>
+        <v>298.616</v>
       </c>
       <c r="P630" t="n">
-        <v>0</v>
+        <v>0.497</v>
       </c>
       <c r="Q630" t="n">
-        <v>0</v>
+        <v>2.841</v>
       </c>
       <c r="R630" t="n">
-        <v>0</v>
+        <v>3.773</v>
       </c>
       <c r="S630" t="n">
-        <v>0</v>
+        <v>31.889</v>
       </c>
       <c r="T630" t="n">
-        <v>0</v>
+        <v>0.048</v>
       </c>
       <c r="U630" t="n">
-        <v>0</v>
+        <v>0.656</v>
       </c>
       <c r="V630" t="n">
-        <v>0</v>
+        <v>0.306</v>
       </c>
       <c r="W630" t="n">
-        <v>0</v>
+        <v>2.021</v>
       </c>
       <c r="X630" t="n">
-        <v>0</v>
+        <v>0.07099999999999999</v>
       </c>
       <c r="Y630" t="n">
-        <v>0</v>
+        <v>0.802</v>
       </c>
       <c r="Z630" t="n">
-        <v>0</v>
+        <v>13.699</v>
       </c>
       <c r="AA630" t="n">
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="AB630" t="n">
-        <v>0</v>
+        <v>29.677</v>
       </c>
       <c r="AC630" t="inlineStr"/>
     </row>
@@ -68821,67 +68349,67 @@
         <v>0</v>
       </c>
       <c r="H631" t="n">
-        <v>0</v>
+        <v>187.375</v>
       </c>
       <c r="I631" t="n">
-        <v>0</v>
+        <v>1.253</v>
       </c>
       <c r="J631" t="n">
-        <v>0</v>
+        <v>11.381</v>
       </c>
       <c r="K631" t="n">
-        <v>0</v>
+        <v>0.137</v>
       </c>
       <c r="L631" t="n">
-        <v>0</v>
+        <v>0.879</v>
       </c>
       <c r="M631" t="n">
-        <v>0</v>
+        <v>0.198</v>
       </c>
       <c r="N631" t="n">
-        <v>0</v>
+        <v>94.255</v>
       </c>
       <c r="O631" t="n">
-        <v>0</v>
+        <v>280.495</v>
       </c>
       <c r="P631" t="n">
-        <v>0</v>
+        <v>0.434</v>
       </c>
       <c r="Q631" t="n">
-        <v>0</v>
+        <v>2.658</v>
       </c>
       <c r="R631" t="n">
-        <v>0</v>
+        <v>3.939</v>
       </c>
       <c r="S631" t="n">
-        <v>0</v>
+        <v>32.369</v>
       </c>
       <c r="T631" t="n">
-        <v>0</v>
+        <v>0.047</v>
       </c>
       <c r="U631" t="n">
-        <v>0</v>
+        <v>0.655</v>
       </c>
       <c r="V631" t="n">
-        <v>0</v>
+        <v>0.304</v>
       </c>
       <c r="W631" t="n">
-        <v>0</v>
+        <v>2.015</v>
       </c>
       <c r="X631" t="n">
-        <v>0</v>
+        <v>0.06900000000000001</v>
       </c>
       <c r="Y631" t="n">
-        <v>0</v>
+        <v>0.796</v>
       </c>
       <c r="Z631" t="n">
-        <v>0</v>
+        <v>12.312</v>
       </c>
       <c r="AA631" t="n">
-        <v>0</v>
+        <v>0.5620000000000001</v>
       </c>
       <c r="AB631" t="n">
-        <v>0</v>
+        <v>28.273</v>
       </c>
       <c r="AC631" t="inlineStr"/>
     </row>

</xml_diff>